<commit_message>
feat: add new attendees to spreadsheet
</commit_message>
<xml_diff>
--- a/data/wg_attendees.xlsx
+++ b/data/wg_attendees.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="189" uniqueCount="189">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="196" uniqueCount="196">
   <si>
     <t>name</t>
   </si>
@@ -584,6 +584,27 @@
   </si>
   <si>
     <t>https://cytel.com/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vinod Kumar</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TruMines Clinical</t>
+  </si>
+  <si>
+    <t>https://trumindsclinical.com/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chi-Hua Huang</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Astellas Pharmaceuticals</t>
+  </si>
+  <si>
+    <t>https://www.astellas.com/en/</t>
+  </si>
+  <si>
+    <t>Ram</t>
   </si>
 </sst>
 </file>
@@ -646,13 +667,13 @@
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyProtection="1">
       <protection hidden="0" locked="1"/>
     </xf>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyProtection="1">
-      <protection hidden="0" locked="1"/>
-    </xf>
     <xf fontId="2" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyProtection="1">
       <protection hidden="0" locked="1"/>
     </xf>
     <xf fontId="3" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyProtection="1">
+      <protection hidden="0" locked="1"/>
+    </xf>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyProtection="1">
       <protection hidden="0" locked="1"/>
     </xf>
   </cellXfs>
@@ -1110,10 +1131,10 @@
       <c r="A2" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="C2" s="3"/>
+      <c r="C2" s="2"/>
     </row>
     <row r="3" ht="12.800000000000001">
       <c r="A3" s="1" t="s">
@@ -1122,7 +1143,7 @@
       <c r="B3" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="C3" s="2" t="s">
         <v>7</v>
       </c>
     </row>
@@ -1133,7 +1154,7 @@
       <c r="B4" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" s="2" t="s">
         <v>7</v>
       </c>
     </row>
@@ -1144,7 +1165,7 @@
       <c r="B5" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="C5" s="2" t="s">
         <v>7</v>
       </c>
     </row>
@@ -1152,10 +1173,10 @@
       <c r="A6" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="B6" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="C6" s="4" t="s">
+      <c r="C6" s="3" t="s">
         <v>12</v>
       </c>
     </row>
@@ -1166,7 +1187,7 @@
       <c r="B7" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C7" s="3" t="s">
+      <c r="C7" s="2" t="s">
         <v>7</v>
       </c>
     </row>
@@ -1177,7 +1198,7 @@
       <c r="B8" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C8" s="3" t="s">
+      <c r="C8" s="2" t="s">
         <v>7</v>
       </c>
     </row>
@@ -1188,7 +1209,7 @@
       <c r="B9" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="C9" s="3" t="s">
+      <c r="C9" s="2" t="s">
         <v>17</v>
       </c>
     </row>
@@ -1199,7 +1220,7 @@
       <c r="B10" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="C10" s="3" t="s">
+      <c r="C10" s="2" t="s">
         <v>17</v>
       </c>
     </row>
@@ -1210,7 +1231,7 @@
       <c r="B11" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="C11" s="3" t="s">
+      <c r="C11" s="2" t="s">
         <v>17</v>
       </c>
     </row>
@@ -1221,7 +1242,7 @@
       <c r="B12" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="C12" s="3" t="s">
+      <c r="C12" s="2" t="s">
         <v>17</v>
       </c>
     </row>
@@ -1232,7 +1253,7 @@
       <c r="B13" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="C13" s="3" t="s">
+      <c r="C13" s="2" t="s">
         <v>23</v>
       </c>
     </row>
@@ -1243,7 +1264,7 @@
       <c r="B14" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="C14" s="3" t="s">
+      <c r="C14" s="2" t="s">
         <v>26</v>
       </c>
     </row>
@@ -1254,7 +1275,7 @@
       <c r="B15" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="C15" s="3" t="s">
+      <c r="C15" s="2" t="s">
         <v>29</v>
       </c>
     </row>
@@ -1265,7 +1286,7 @@
       <c r="B16" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="C16" s="3" t="s">
+      <c r="C16" s="2" t="s">
         <v>29</v>
       </c>
     </row>
@@ -1276,7 +1297,7 @@
       <c r="B17" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="C17" s="3" t="s">
+      <c r="C17" s="2" t="s">
         <v>33</v>
       </c>
     </row>
@@ -1287,7 +1308,7 @@
       <c r="B18" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="C18" s="3" t="s">
+      <c r="C18" s="2" t="s">
         <v>33</v>
       </c>
     </row>
@@ -1298,7 +1319,7 @@
       <c r="B19" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="C19" s="3" t="s">
+      <c r="C19" s="2" t="s">
         <v>33</v>
       </c>
     </row>
@@ -1309,7 +1330,7 @@
       <c r="B20" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="C20" s="3" t="s">
+      <c r="C20" s="2" t="s">
         <v>33</v>
       </c>
     </row>
@@ -1320,7 +1341,7 @@
       <c r="B21" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="C21" s="3" t="s">
+      <c r="C21" s="2" t="s">
         <v>33</v>
       </c>
     </row>
@@ -1331,18 +1352,18 @@
       <c r="B22" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="C22" s="3" t="s">
+      <c r="C22" s="2" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="23" ht="12.800000000000001">
-      <c r="A23" s="2" t="s">
+      <c r="A23" s="1" t="s">
         <v>39</v>
       </c>
       <c r="B23" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="C23" s="3" t="s">
+      <c r="C23" s="2" t="s">
         <v>33</v>
       </c>
     </row>
@@ -1353,7 +1374,7 @@
       <c r="B24" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="C24" s="3" t="s">
+      <c r="C24" s="2" t="s">
         <v>33</v>
       </c>
     </row>
@@ -1364,7 +1385,7 @@
       <c r="B25" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="C25" s="3" t="s">
+      <c r="C25" s="2" t="s">
         <v>43</v>
       </c>
     </row>
@@ -1375,7 +1396,7 @@
       <c r="B26" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="C26" s="3" t="s">
+      <c r="C26" s="2" t="s">
         <v>46</v>
       </c>
     </row>
@@ -1386,7 +1407,7 @@
       <c r="B27" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="C27" s="3" t="s">
+      <c r="C27" s="2" t="s">
         <v>49</v>
       </c>
     </row>
@@ -1397,7 +1418,7 @@
       <c r="B28" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="C28" s="3" t="s">
+      <c r="C28" s="2" t="s">
         <v>52</v>
       </c>
     </row>
@@ -1408,7 +1429,7 @@
       <c r="B29" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="C29" s="3" t="s">
+      <c r="C29" s="2" t="s">
         <v>52</v>
       </c>
     </row>
@@ -1419,7 +1440,7 @@
       <c r="B30" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="C30" s="3" t="s">
+      <c r="C30" s="2" t="s">
         <v>56</v>
       </c>
     </row>
@@ -1430,7 +1451,7 @@
       <c r="B31" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="C31" s="3" t="s">
+      <c r="C31" s="2" t="s">
         <v>52</v>
       </c>
     </row>
@@ -1441,7 +1462,7 @@
       <c r="B32" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="C32" s="3" t="s">
+      <c r="C32" s="2" t="s">
         <v>52</v>
       </c>
     </row>
@@ -1452,7 +1473,7 @@
       <c r="B33" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="C33" s="3" t="s">
+      <c r="C33" s="2" t="s">
         <v>61</v>
       </c>
     </row>
@@ -1463,7 +1484,7 @@
       <c r="B34" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="C34" s="3" t="s">
+      <c r="C34" s="2" t="s">
         <v>64</v>
       </c>
     </row>
@@ -1474,7 +1495,7 @@
       <c r="B35" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="C35" s="3" t="s">
+      <c r="C35" s="2" t="s">
         <v>64</v>
       </c>
     </row>
@@ -1485,7 +1506,7 @@
       <c r="B36" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="C36" s="3" t="s">
+      <c r="C36" s="2" t="s">
         <v>64</v>
       </c>
     </row>
@@ -1496,7 +1517,7 @@
       <c r="B37" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="C37" s="3" t="s">
+      <c r="C37" s="2" t="s">
         <v>64</v>
       </c>
     </row>
@@ -1507,7 +1528,7 @@
       <c r="B38" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="C38" s="3" t="s">
+      <c r="C38" s="2" t="s">
         <v>70</v>
       </c>
     </row>
@@ -1518,7 +1539,7 @@
       <c r="B39" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="C39" s="3" t="s">
+      <c r="C39" s="2" t="s">
         <v>73</v>
       </c>
     </row>
@@ -1529,7 +1550,7 @@
       <c r="B40" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="C40" s="3" t="s">
+      <c r="C40" s="2" t="s">
         <v>76</v>
       </c>
     </row>
@@ -1540,7 +1561,7 @@
       <c r="B41" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="C41" s="3" t="s">
+      <c r="C41" s="2" t="s">
         <v>79</v>
       </c>
     </row>
@@ -1551,7 +1572,7 @@
       <c r="B42" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="C42" s="3" t="s">
+      <c r="C42" s="2" t="s">
         <v>79</v>
       </c>
     </row>
@@ -1562,7 +1583,7 @@
       <c r="B43" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="C43" s="3" t="s">
+      <c r="C43" s="2" t="s">
         <v>79</v>
       </c>
     </row>
@@ -1573,7 +1594,7 @@
       <c r="B44" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="C44" s="3" t="s">
+      <c r="C44" s="2" t="s">
         <v>84</v>
       </c>
     </row>
@@ -1584,7 +1605,7 @@
       <c r="B45" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="C45" s="3" t="s">
+      <c r="C45" s="2" t="s">
         <v>87</v>
       </c>
     </row>
@@ -1595,7 +1616,7 @@
       <c r="B46" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="C46" s="3" t="s">
+      <c r="C46" s="2" t="s">
         <v>90</v>
       </c>
     </row>
@@ -1606,7 +1627,7 @@
       <c r="B47" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="C47" s="3" t="s">
+      <c r="C47" s="2" t="s">
         <v>79</v>
       </c>
     </row>
@@ -1617,7 +1638,7 @@
       <c r="B48" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="C48" s="3" t="s">
+      <c r="C48" s="2" t="s">
         <v>93</v>
       </c>
     </row>
@@ -1628,7 +1649,7 @@
       <c r="B49" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="C49" s="3" t="s">
+      <c r="C49" s="2" t="s">
         <v>33</v>
       </c>
     </row>
@@ -1639,7 +1660,7 @@
       <c r="B50" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="C50" s="3" t="s">
+      <c r="C50" s="2" t="s">
         <v>61</v>
       </c>
     </row>
@@ -1650,7 +1671,7 @@
       <c r="B51" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="C51" s="3" t="s">
+      <c r="C51" s="2" t="s">
         <v>90</v>
       </c>
     </row>
@@ -1661,7 +1682,7 @@
       <c r="B52" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="C52" s="3" t="s">
+      <c r="C52" s="2" t="s">
         <v>33</v>
       </c>
     </row>
@@ -1672,7 +1693,7 @@
       <c r="B53" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="C53" s="3" t="s">
+      <c r="C53" s="2" t="s">
         <v>100</v>
       </c>
     </row>
@@ -1683,7 +1704,7 @@
       <c r="B54" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="C54" s="3" t="s">
+      <c r="C54" s="2" t="s">
         <v>93</v>
       </c>
     </row>
@@ -1694,7 +1715,7 @@
       <c r="B55" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="C55" s="3" t="s">
+      <c r="C55" s="2" t="s">
         <v>79</v>
       </c>
     </row>
@@ -1705,7 +1726,7 @@
       <c r="B56" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="C56" s="3" t="s">
+      <c r="C56" s="2" t="s">
         <v>90</v>
       </c>
     </row>
@@ -1716,7 +1737,7 @@
       <c r="B57" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C57" s="3" t="s">
+      <c r="C57" s="2" t="s">
         <v>7</v>
       </c>
     </row>
@@ -1727,7 +1748,7 @@
       <c r="B58" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="C58" s="3" t="s">
+      <c r="C58" s="2" t="s">
         <v>107</v>
       </c>
     </row>
@@ -1738,7 +1759,7 @@
       <c r="B59" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C59" s="3" t="s">
+      <c r="C59" s="2" t="s">
         <v>7</v>
       </c>
     </row>
@@ -1749,7 +1770,7 @@
       <c r="B60" s="1" t="s">
         <v>110</v>
       </c>
-      <c r="C60" s="3" t="s">
+      <c r="C60" s="2" t="s">
         <v>111</v>
       </c>
     </row>
@@ -1768,7 +1789,7 @@
       <c r="B62" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="C62" s="3" t="s">
+      <c r="C62" s="2" t="s">
         <v>115</v>
       </c>
     </row>
@@ -1779,7 +1800,7 @@
       <c r="B63" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="C63" s="3" t="s">
+      <c r="C63" s="2" t="s">
         <v>107</v>
       </c>
     </row>
@@ -1790,7 +1811,7 @@
       <c r="B64" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C64" s="3" t="s">
+      <c r="C64" s="2" t="s">
         <v>7</v>
       </c>
     </row>
@@ -1801,7 +1822,7 @@
       <c r="B65" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="C65" s="3" t="s">
+      <c r="C65" s="2" t="s">
         <v>107</v>
       </c>
     </row>
@@ -1812,7 +1833,7 @@
       <c r="B66" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="C66" s="3" t="s">
+      <c r="C66" s="2" t="s">
         <v>121</v>
       </c>
     </row>
@@ -1823,7 +1844,7 @@
       <c r="B67" s="1" t="s">
         <v>110</v>
       </c>
-      <c r="C67" s="3" t="s">
+      <c r="C67" s="2" t="s">
         <v>111</v>
       </c>
     </row>
@@ -1834,7 +1855,7 @@
       <c r="B68" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C68" s="3" t="s">
+      <c r="C68" s="2" t="s">
         <v>7</v>
       </c>
     </row>
@@ -1845,7 +1866,7 @@
       <c r="B69" s="1" t="s">
         <v>125</v>
       </c>
-      <c r="C69" s="3" t="s">
+      <c r="C69" s="2" t="s">
         <v>126</v>
       </c>
     </row>
@@ -1856,7 +1877,7 @@
       <c r="B70" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="C70" s="3" t="s">
+      <c r="C70" s="2" t="s">
         <v>33</v>
       </c>
     </row>
@@ -1867,7 +1888,7 @@
       <c r="B71" s="1" t="s">
         <v>110</v>
       </c>
-      <c r="C71" s="3" t="s">
+      <c r="C71" s="2" t="s">
         <v>111</v>
       </c>
     </row>
@@ -1878,7 +1899,7 @@
       <c r="B72" s="1" t="s">
         <v>130</v>
       </c>
-      <c r="C72" s="3" t="s">
+      <c r="C72" s="2" t="s">
         <v>131</v>
       </c>
     </row>
@@ -1889,7 +1910,7 @@
       <c r="B73" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="C73" s="3" t="s">
+      <c r="C73" s="2" t="s">
         <v>43</v>
       </c>
     </row>
@@ -1900,7 +1921,7 @@
       <c r="B74" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="C74" s="3" t="s">
+      <c r="C74" s="2" t="s">
         <v>43</v>
       </c>
     </row>
@@ -1911,7 +1932,7 @@
       <c r="B75" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="C75" s="3" t="s">
+      <c r="C75" s="2" t="s">
         <v>52</v>
       </c>
     </row>
@@ -1922,7 +1943,7 @@
       <c r="B76" s="1" t="s">
         <v>136</v>
       </c>
-      <c r="C76" s="3" t="s">
+      <c r="C76" s="2" t="s">
         <v>137</v>
       </c>
     </row>
@@ -1933,7 +1954,7 @@
       <c r="B77" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C77" s="3" t="s">
+      <c r="C77" s="2" t="s">
         <v>7</v>
       </c>
     </row>
@@ -1944,7 +1965,7 @@
       <c r="B78" s="1" t="s">
         <v>140</v>
       </c>
-      <c r="C78" s="3" t="s">
+      <c r="C78" s="2" t="s">
         <v>141</v>
       </c>
     </row>
@@ -1955,7 +1976,7 @@
       <c r="B79" s="1" t="s">
         <v>143</v>
       </c>
-      <c r="C79" s="3" t="s">
+      <c r="C79" s="2" t="s">
         <v>144</v>
       </c>
     </row>
@@ -1966,7 +1987,7 @@
       <c r="B80" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C80" s="3" t="s">
+      <c r="C80" s="2" t="s">
         <v>7</v>
       </c>
     </row>
@@ -1977,7 +1998,7 @@
       <c r="B81" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="C81" s="3" t="s">
+      <c r="C81" s="2" t="s">
         <v>84</v>
       </c>
     </row>
@@ -1988,7 +2009,7 @@
       <c r="B82" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="C82" s="3" t="s">
+      <c r="C82" s="2" t="s">
         <v>64</v>
       </c>
     </row>
@@ -1999,7 +2020,7 @@
       <c r="B83" s="1" t="s">
         <v>149</v>
       </c>
-      <c r="C83" s="3" t="s">
+      <c r="C83" s="2" t="s">
         <v>150</v>
       </c>
     </row>
@@ -2010,7 +2031,7 @@
       <c r="B84" s="1" t="s">
         <v>152</v>
       </c>
-      <c r="C84" s="3" t="s">
+      <c r="C84" s="2" t="s">
         <v>153</v>
       </c>
     </row>
@@ -2021,7 +2042,7 @@
       <c r="B85" s="1" t="s">
         <v>140</v>
       </c>
-      <c r="C85" s="3" t="s">
+      <c r="C85" s="2" t="s">
         <v>141</v>
       </c>
     </row>
@@ -2032,7 +2053,7 @@
       <c r="B86" s="1" t="s">
         <v>140</v>
       </c>
-      <c r="C86" s="3" t="s">
+      <c r="C86" s="2" t="s">
         <v>141</v>
       </c>
     </row>
@@ -2043,7 +2064,7 @@
       <c r="B87" s="1" t="s">
         <v>157</v>
       </c>
-      <c r="C87" s="3" t="s">
+      <c r="C87" s="2" t="s">
         <v>158</v>
       </c>
     </row>
@@ -2054,7 +2075,7 @@
       <c r="B88" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="C88" s="3" t="s">
+      <c r="C88" s="2" t="s">
         <v>79</v>
       </c>
     </row>
@@ -2065,7 +2086,7 @@
       <c r="B89" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="C89" s="3" t="s">
+      <c r="C89" s="2" t="s">
         <v>87</v>
       </c>
     </row>
@@ -2076,7 +2097,7 @@
       <c r="B90" s="1" t="s">
         <v>162</v>
       </c>
-      <c r="C90" s="3" t="s">
+      <c r="C90" s="2" t="s">
         <v>163</v>
       </c>
     </row>
@@ -2087,7 +2108,7 @@
       <c r="B91" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="C91" s="3" t="s">
+      <c r="C91" s="2" t="s">
         <v>33</v>
       </c>
     </row>
@@ -2098,7 +2119,7 @@
       <c r="B92" s="1" t="s">
         <v>166</v>
       </c>
-      <c r="C92" s="3" t="s">
+      <c r="C92" s="2" t="s">
         <v>167</v>
       </c>
     </row>
@@ -2109,7 +2130,7 @@
       <c r="B93" s="1" t="s">
         <v>169</v>
       </c>
-      <c r="C93" s="3" t="s">
+      <c r="C93" s="2" t="s">
         <v>170</v>
       </c>
     </row>
@@ -2128,101 +2149,131 @@
       <c r="B95" s="1" t="s">
         <v>174</v>
       </c>
-      <c r="C95" s="3" t="s">
+      <c r="C95" s="2" t="s">
         <v>175</v>
       </c>
     </row>
     <row r="96" ht="15">
-      <c r="A96" s="2" t="s">
+      <c r="A96" s="1" t="s">
         <v>176</v>
       </c>
-      <c r="B96" s="2" t="s">
+      <c r="B96" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="C96" s="3" t="s">
+      <c r="C96" s="2" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="97" ht="15">
-      <c r="A97" s="2" t="s">
+      <c r="A97" s="1" t="s">
         <v>177</v>
       </c>
-      <c r="B97" s="2" t="s">
+      <c r="B97" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="C97" s="4" t="s">
+      <c r="C97" s="3" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="98" ht="15">
-      <c r="A98" s="2" t="s">
+      <c r="A98" s="1" t="s">
         <v>178</v>
       </c>
-      <c r="B98" s="2" t="s">
+      <c r="B98" s="1" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="99" ht="15">
-      <c r="A99" s="2" t="s">
+      <c r="A99" s="1" t="s">
         <v>179</v>
       </c>
-      <c r="B99" s="2" t="s">
+      <c r="B99" s="1" t="s">
         <v>180</v>
       </c>
-      <c r="C99" s="4" t="s">
+      <c r="C99" s="3" t="s">
         <v>181</v>
       </c>
     </row>
     <row r="100" ht="15">
-      <c r="A100" s="2" t="s">
+      <c r="A100" s="1" t="s">
         <v>182</v>
       </c>
-      <c r="B100" s="2" t="s">
+      <c r="B100" s="1" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="101" ht="15">
-      <c r="A101" s="2" t="s">
+      <c r="A101" s="1" t="s">
         <v>183</v>
       </c>
-      <c r="B101" s="2" t="s">
+      <c r="B101" s="1" t="s">
         <v>110</v>
       </c>
-      <c r="C101" s="3" t="s">
+      <c r="C101" s="2" t="s">
         <v>111</v>
       </c>
     </row>
     <row r="102" ht="15">
-      <c r="A102" s="2" t="s">
+      <c r="A102" s="1" t="s">
         <v>184</v>
       </c>
-      <c r="B102" s="2" t="s">
+      <c r="B102" s="1" t="s">
         <v>149</v>
       </c>
-      <c r="C102" s="3" t="s">
+      <c r="C102" s="2" t="s">
         <v>150</v>
       </c>
     </row>
     <row r="103" ht="15">
-      <c r="A103" s="2" t="s">
+      <c r="A103" s="1" t="s">
         <v>185</v>
       </c>
-      <c r="B103" s="2" t="s">
+      <c r="B103" s="1" t="s">
         <v>110</v>
       </c>
-      <c r="C103" s="3" t="s">
+      <c r="C103" s="2" t="s">
         <v>111</v>
       </c>
     </row>
     <row r="104" ht="15">
-      <c r="A104" s="2" t="s">
+      <c r="A104" s="1" t="s">
         <v>186</v>
       </c>
-      <c r="B104" s="2" t="s">
+      <c r="B104" s="1" t="s">
         <v>187</v>
       </c>
-      <c r="C104" s="4" t="s">
+      <c r="C104" s="3" t="s">
         <v>188</v>
+      </c>
+    </row>
+    <row r="105" ht="15">
+      <c r="A105" s="4" t="s">
+        <v>189</v>
+      </c>
+      <c r="B105" s="4" t="s">
+        <v>190</v>
+      </c>
+      <c r="C105" s="3" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="106" ht="15">
+      <c r="A106" s="4" t="s">
+        <v>192</v>
+      </c>
+      <c r="B106" s="4" t="s">
+        <v>193</v>
+      </c>
+      <c r="C106" s="3" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="107" ht="15">
+      <c r="A107" s="4" t="s">
+        <v>195</v>
+      </c>
+      <c r="B107" s="4" t="s">
+        <v>4</v>
       </c>
     </row>
   </sheetData>
@@ -2325,6 +2376,8 @@
     <hyperlink r:id="rId32" ref="C102"/>
     <hyperlink r:id="rId24" ref="C103"/>
     <hyperlink r:id="rId40" ref="C104"/>
+    <hyperlink r:id="rId41" ref="C105"/>
+    <hyperlink r:id="rId42" ref="C106"/>
   </hyperlinks>
   <printOptions headings="0" gridLines="0" horizontalCentered="0" verticalCentered="0"/>
   <pageMargins left="0.78750000000000009" right="0.78750000000000009" top="1.05277777777778" bottom="1.05277777777778" header="0.78750000000000009" footer="0.78750000000000009"/>

</xml_diff>

<commit_message>
Minutes 2026 03 06 (#169)
* feat: add new attendees to spreadsheet

* fix: update minutes template to include AI summary disclaimer

* feat: minutes for 2026-03-06

* fix: add links from chat and summary of AI discussion
</commit_message>
<xml_diff>
--- a/data/wg_attendees.xlsx
+++ b/data/wg_attendees.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="189" uniqueCount="189">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="196" uniqueCount="196">
   <si>
     <t>name</t>
   </si>
@@ -584,6 +584,27 @@
   </si>
   <si>
     <t>https://cytel.com/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vinod Kumar</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TruMines Clinical</t>
+  </si>
+  <si>
+    <t>https://trumindsclinical.com/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chi-Hua Huang</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Astellas Pharmaceuticals</t>
+  </si>
+  <si>
+    <t>https://www.astellas.com/en/</t>
+  </si>
+  <si>
+    <t>Ram</t>
   </si>
 </sst>
 </file>
@@ -646,13 +667,13 @@
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyProtection="1">
       <protection hidden="0" locked="1"/>
     </xf>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyProtection="1">
-      <protection hidden="0" locked="1"/>
-    </xf>
     <xf fontId="2" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyProtection="1">
       <protection hidden="0" locked="1"/>
     </xf>
     <xf fontId="3" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyProtection="1">
+      <protection hidden="0" locked="1"/>
+    </xf>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyProtection="1">
       <protection hidden="0" locked="1"/>
     </xf>
   </cellXfs>
@@ -1110,10 +1131,10 @@
       <c r="A2" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="C2" s="3"/>
+      <c r="C2" s="2"/>
     </row>
     <row r="3" ht="12.800000000000001">
       <c r="A3" s="1" t="s">
@@ -1122,7 +1143,7 @@
       <c r="B3" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="C3" s="2" t="s">
         <v>7</v>
       </c>
     </row>
@@ -1133,7 +1154,7 @@
       <c r="B4" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" s="2" t="s">
         <v>7</v>
       </c>
     </row>
@@ -1144,7 +1165,7 @@
       <c r="B5" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="C5" s="2" t="s">
         <v>7</v>
       </c>
     </row>
@@ -1152,10 +1173,10 @@
       <c r="A6" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="B6" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="C6" s="4" t="s">
+      <c r="C6" s="3" t="s">
         <v>12</v>
       </c>
     </row>
@@ -1166,7 +1187,7 @@
       <c r="B7" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C7" s="3" t="s">
+      <c r="C7" s="2" t="s">
         <v>7</v>
       </c>
     </row>
@@ -1177,7 +1198,7 @@
       <c r="B8" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C8" s="3" t="s">
+      <c r="C8" s="2" t="s">
         <v>7</v>
       </c>
     </row>
@@ -1188,7 +1209,7 @@
       <c r="B9" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="C9" s="3" t="s">
+      <c r="C9" s="2" t="s">
         <v>17</v>
       </c>
     </row>
@@ -1199,7 +1220,7 @@
       <c r="B10" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="C10" s="3" t="s">
+      <c r="C10" s="2" t="s">
         <v>17</v>
       </c>
     </row>
@@ -1210,7 +1231,7 @@
       <c r="B11" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="C11" s="3" t="s">
+      <c r="C11" s="2" t="s">
         <v>17</v>
       </c>
     </row>
@@ -1221,7 +1242,7 @@
       <c r="B12" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="C12" s="3" t="s">
+      <c r="C12" s="2" t="s">
         <v>17</v>
       </c>
     </row>
@@ -1232,7 +1253,7 @@
       <c r="B13" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="C13" s="3" t="s">
+      <c r="C13" s="2" t="s">
         <v>23</v>
       </c>
     </row>
@@ -1243,7 +1264,7 @@
       <c r="B14" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="C14" s="3" t="s">
+      <c r="C14" s="2" t="s">
         <v>26</v>
       </c>
     </row>
@@ -1254,7 +1275,7 @@
       <c r="B15" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="C15" s="3" t="s">
+      <c r="C15" s="2" t="s">
         <v>29</v>
       </c>
     </row>
@@ -1265,7 +1286,7 @@
       <c r="B16" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="C16" s="3" t="s">
+      <c r="C16" s="2" t="s">
         <v>29</v>
       </c>
     </row>
@@ -1276,7 +1297,7 @@
       <c r="B17" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="C17" s="3" t="s">
+      <c r="C17" s="2" t="s">
         <v>33</v>
       </c>
     </row>
@@ -1287,7 +1308,7 @@
       <c r="B18" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="C18" s="3" t="s">
+      <c r="C18" s="2" t="s">
         <v>33</v>
       </c>
     </row>
@@ -1298,7 +1319,7 @@
       <c r="B19" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="C19" s="3" t="s">
+      <c r="C19" s="2" t="s">
         <v>33</v>
       </c>
     </row>
@@ -1309,7 +1330,7 @@
       <c r="B20" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="C20" s="3" t="s">
+      <c r="C20" s="2" t="s">
         <v>33</v>
       </c>
     </row>
@@ -1320,7 +1341,7 @@
       <c r="B21" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="C21" s="3" t="s">
+      <c r="C21" s="2" t="s">
         <v>33</v>
       </c>
     </row>
@@ -1331,18 +1352,18 @@
       <c r="B22" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="C22" s="3" t="s">
+      <c r="C22" s="2" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="23" ht="12.800000000000001">
-      <c r="A23" s="2" t="s">
+      <c r="A23" s="1" t="s">
         <v>39</v>
       </c>
       <c r="B23" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="C23" s="3" t="s">
+      <c r="C23" s="2" t="s">
         <v>33</v>
       </c>
     </row>
@@ -1353,7 +1374,7 @@
       <c r="B24" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="C24" s="3" t="s">
+      <c r="C24" s="2" t="s">
         <v>33</v>
       </c>
     </row>
@@ -1364,7 +1385,7 @@
       <c r="B25" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="C25" s="3" t="s">
+      <c r="C25" s="2" t="s">
         <v>43</v>
       </c>
     </row>
@@ -1375,7 +1396,7 @@
       <c r="B26" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="C26" s="3" t="s">
+      <c r="C26" s="2" t="s">
         <v>46</v>
       </c>
     </row>
@@ -1386,7 +1407,7 @@
       <c r="B27" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="C27" s="3" t="s">
+      <c r="C27" s="2" t="s">
         <v>49</v>
       </c>
     </row>
@@ -1397,7 +1418,7 @@
       <c r="B28" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="C28" s="3" t="s">
+      <c r="C28" s="2" t="s">
         <v>52</v>
       </c>
     </row>
@@ -1408,7 +1429,7 @@
       <c r="B29" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="C29" s="3" t="s">
+      <c r="C29" s="2" t="s">
         <v>52</v>
       </c>
     </row>
@@ -1419,7 +1440,7 @@
       <c r="B30" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="C30" s="3" t="s">
+      <c r="C30" s="2" t="s">
         <v>56</v>
       </c>
     </row>
@@ -1430,7 +1451,7 @@
       <c r="B31" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="C31" s="3" t="s">
+      <c r="C31" s="2" t="s">
         <v>52</v>
       </c>
     </row>
@@ -1441,7 +1462,7 @@
       <c r="B32" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="C32" s="3" t="s">
+      <c r="C32" s="2" t="s">
         <v>52</v>
       </c>
     </row>
@@ -1452,7 +1473,7 @@
       <c r="B33" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="C33" s="3" t="s">
+      <c r="C33" s="2" t="s">
         <v>61</v>
       </c>
     </row>
@@ -1463,7 +1484,7 @@
       <c r="B34" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="C34" s="3" t="s">
+      <c r="C34" s="2" t="s">
         <v>64</v>
       </c>
     </row>
@@ -1474,7 +1495,7 @@
       <c r="B35" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="C35" s="3" t="s">
+      <c r="C35" s="2" t="s">
         <v>64</v>
       </c>
     </row>
@@ -1485,7 +1506,7 @@
       <c r="B36" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="C36" s="3" t="s">
+      <c r="C36" s="2" t="s">
         <v>64</v>
       </c>
     </row>
@@ -1496,7 +1517,7 @@
       <c r="B37" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="C37" s="3" t="s">
+      <c r="C37" s="2" t="s">
         <v>64</v>
       </c>
     </row>
@@ -1507,7 +1528,7 @@
       <c r="B38" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="C38" s="3" t="s">
+      <c r="C38" s="2" t="s">
         <v>70</v>
       </c>
     </row>
@@ -1518,7 +1539,7 @@
       <c r="B39" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="C39" s="3" t="s">
+      <c r="C39" s="2" t="s">
         <v>73</v>
       </c>
     </row>
@@ -1529,7 +1550,7 @@
       <c r="B40" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="C40" s="3" t="s">
+      <c r="C40" s="2" t="s">
         <v>76</v>
       </c>
     </row>
@@ -1540,7 +1561,7 @@
       <c r="B41" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="C41" s="3" t="s">
+      <c r="C41" s="2" t="s">
         <v>79</v>
       </c>
     </row>
@@ -1551,7 +1572,7 @@
       <c r="B42" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="C42" s="3" t="s">
+      <c r="C42" s="2" t="s">
         <v>79</v>
       </c>
     </row>
@@ -1562,7 +1583,7 @@
       <c r="B43" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="C43" s="3" t="s">
+      <c r="C43" s="2" t="s">
         <v>79</v>
       </c>
     </row>
@@ -1573,7 +1594,7 @@
       <c r="B44" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="C44" s="3" t="s">
+      <c r="C44" s="2" t="s">
         <v>84</v>
       </c>
     </row>
@@ -1584,7 +1605,7 @@
       <c r="B45" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="C45" s="3" t="s">
+      <c r="C45" s="2" t="s">
         <v>87</v>
       </c>
     </row>
@@ -1595,7 +1616,7 @@
       <c r="B46" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="C46" s="3" t="s">
+      <c r="C46" s="2" t="s">
         <v>90</v>
       </c>
     </row>
@@ -1606,7 +1627,7 @@
       <c r="B47" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="C47" s="3" t="s">
+      <c r="C47" s="2" t="s">
         <v>79</v>
       </c>
     </row>
@@ -1617,7 +1638,7 @@
       <c r="B48" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="C48" s="3" t="s">
+      <c r="C48" s="2" t="s">
         <v>93</v>
       </c>
     </row>
@@ -1628,7 +1649,7 @@
       <c r="B49" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="C49" s="3" t="s">
+      <c r="C49" s="2" t="s">
         <v>33</v>
       </c>
     </row>
@@ -1639,7 +1660,7 @@
       <c r="B50" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="C50" s="3" t="s">
+      <c r="C50" s="2" t="s">
         <v>61</v>
       </c>
     </row>
@@ -1650,7 +1671,7 @@
       <c r="B51" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="C51" s="3" t="s">
+      <c r="C51" s="2" t="s">
         <v>90</v>
       </c>
     </row>
@@ -1661,7 +1682,7 @@
       <c r="B52" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="C52" s="3" t="s">
+      <c r="C52" s="2" t="s">
         <v>33</v>
       </c>
     </row>
@@ -1672,7 +1693,7 @@
       <c r="B53" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="C53" s="3" t="s">
+      <c r="C53" s="2" t="s">
         <v>100</v>
       </c>
     </row>
@@ -1683,7 +1704,7 @@
       <c r="B54" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="C54" s="3" t="s">
+      <c r="C54" s="2" t="s">
         <v>93</v>
       </c>
     </row>
@@ -1694,7 +1715,7 @@
       <c r="B55" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="C55" s="3" t="s">
+      <c r="C55" s="2" t="s">
         <v>79</v>
       </c>
     </row>
@@ -1705,7 +1726,7 @@
       <c r="B56" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="C56" s="3" t="s">
+      <c r="C56" s="2" t="s">
         <v>90</v>
       </c>
     </row>
@@ -1716,7 +1737,7 @@
       <c r="B57" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C57" s="3" t="s">
+      <c r="C57" s="2" t="s">
         <v>7</v>
       </c>
     </row>
@@ -1727,7 +1748,7 @@
       <c r="B58" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="C58" s="3" t="s">
+      <c r="C58" s="2" t="s">
         <v>107</v>
       </c>
     </row>
@@ -1738,7 +1759,7 @@
       <c r="B59" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C59" s="3" t="s">
+      <c r="C59" s="2" t="s">
         <v>7</v>
       </c>
     </row>
@@ -1749,7 +1770,7 @@
       <c r="B60" s="1" t="s">
         <v>110</v>
       </c>
-      <c r="C60" s="3" t="s">
+      <c r="C60" s="2" t="s">
         <v>111</v>
       </c>
     </row>
@@ -1768,7 +1789,7 @@
       <c r="B62" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="C62" s="3" t="s">
+      <c r="C62" s="2" t="s">
         <v>115</v>
       </c>
     </row>
@@ -1779,7 +1800,7 @@
       <c r="B63" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="C63" s="3" t="s">
+      <c r="C63" s="2" t="s">
         <v>107</v>
       </c>
     </row>
@@ -1790,7 +1811,7 @@
       <c r="B64" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C64" s="3" t="s">
+      <c r="C64" s="2" t="s">
         <v>7</v>
       </c>
     </row>
@@ -1801,7 +1822,7 @@
       <c r="B65" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="C65" s="3" t="s">
+      <c r="C65" s="2" t="s">
         <v>107</v>
       </c>
     </row>
@@ -1812,7 +1833,7 @@
       <c r="B66" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="C66" s="3" t="s">
+      <c r="C66" s="2" t="s">
         <v>121</v>
       </c>
     </row>
@@ -1823,7 +1844,7 @@
       <c r="B67" s="1" t="s">
         <v>110</v>
       </c>
-      <c r="C67" s="3" t="s">
+      <c r="C67" s="2" t="s">
         <v>111</v>
       </c>
     </row>
@@ -1834,7 +1855,7 @@
       <c r="B68" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C68" s="3" t="s">
+      <c r="C68" s="2" t="s">
         <v>7</v>
       </c>
     </row>
@@ -1845,7 +1866,7 @@
       <c r="B69" s="1" t="s">
         <v>125</v>
       </c>
-      <c r="C69" s="3" t="s">
+      <c r="C69" s="2" t="s">
         <v>126</v>
       </c>
     </row>
@@ -1856,7 +1877,7 @@
       <c r="B70" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="C70" s="3" t="s">
+      <c r="C70" s="2" t="s">
         <v>33</v>
       </c>
     </row>
@@ -1867,7 +1888,7 @@
       <c r="B71" s="1" t="s">
         <v>110</v>
       </c>
-      <c r="C71" s="3" t="s">
+      <c r="C71" s="2" t="s">
         <v>111</v>
       </c>
     </row>
@@ -1878,7 +1899,7 @@
       <c r="B72" s="1" t="s">
         <v>130</v>
       </c>
-      <c r="C72" s="3" t="s">
+      <c r="C72" s="2" t="s">
         <v>131</v>
       </c>
     </row>
@@ -1889,7 +1910,7 @@
       <c r="B73" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="C73" s="3" t="s">
+      <c r="C73" s="2" t="s">
         <v>43</v>
       </c>
     </row>
@@ -1900,7 +1921,7 @@
       <c r="B74" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="C74" s="3" t="s">
+      <c r="C74" s="2" t="s">
         <v>43</v>
       </c>
     </row>
@@ -1911,7 +1932,7 @@
       <c r="B75" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="C75" s="3" t="s">
+      <c r="C75" s="2" t="s">
         <v>52</v>
       </c>
     </row>
@@ -1922,7 +1943,7 @@
       <c r="B76" s="1" t="s">
         <v>136</v>
       </c>
-      <c r="C76" s="3" t="s">
+      <c r="C76" s="2" t="s">
         <v>137</v>
       </c>
     </row>
@@ -1933,7 +1954,7 @@
       <c r="B77" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C77" s="3" t="s">
+      <c r="C77" s="2" t="s">
         <v>7</v>
       </c>
     </row>
@@ -1944,7 +1965,7 @@
       <c r="B78" s="1" t="s">
         <v>140</v>
       </c>
-      <c r="C78" s="3" t="s">
+      <c r="C78" s="2" t="s">
         <v>141</v>
       </c>
     </row>
@@ -1955,7 +1976,7 @@
       <c r="B79" s="1" t="s">
         <v>143</v>
       </c>
-      <c r="C79" s="3" t="s">
+      <c r="C79" s="2" t="s">
         <v>144</v>
       </c>
     </row>
@@ -1966,7 +1987,7 @@
       <c r="B80" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C80" s="3" t="s">
+      <c r="C80" s="2" t="s">
         <v>7</v>
       </c>
     </row>
@@ -1977,7 +1998,7 @@
       <c r="B81" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="C81" s="3" t="s">
+      <c r="C81" s="2" t="s">
         <v>84</v>
       </c>
     </row>
@@ -1988,7 +2009,7 @@
       <c r="B82" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="C82" s="3" t="s">
+      <c r="C82" s="2" t="s">
         <v>64</v>
       </c>
     </row>
@@ -1999,7 +2020,7 @@
       <c r="B83" s="1" t="s">
         <v>149</v>
       </c>
-      <c r="C83" s="3" t="s">
+      <c r="C83" s="2" t="s">
         <v>150</v>
       </c>
     </row>
@@ -2010,7 +2031,7 @@
       <c r="B84" s="1" t="s">
         <v>152</v>
       </c>
-      <c r="C84" s="3" t="s">
+      <c r="C84" s="2" t="s">
         <v>153</v>
       </c>
     </row>
@@ -2021,7 +2042,7 @@
       <c r="B85" s="1" t="s">
         <v>140</v>
       </c>
-      <c r="C85" s="3" t="s">
+      <c r="C85" s="2" t="s">
         <v>141</v>
       </c>
     </row>
@@ -2032,7 +2053,7 @@
       <c r="B86" s="1" t="s">
         <v>140</v>
       </c>
-      <c r="C86" s="3" t="s">
+      <c r="C86" s="2" t="s">
         <v>141</v>
       </c>
     </row>
@@ -2043,7 +2064,7 @@
       <c r="B87" s="1" t="s">
         <v>157</v>
       </c>
-      <c r="C87" s="3" t="s">
+      <c r="C87" s="2" t="s">
         <v>158</v>
       </c>
     </row>
@@ -2054,7 +2075,7 @@
       <c r="B88" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="C88" s="3" t="s">
+      <c r="C88" s="2" t="s">
         <v>79</v>
       </c>
     </row>
@@ -2065,7 +2086,7 @@
       <c r="B89" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="C89" s="3" t="s">
+      <c r="C89" s="2" t="s">
         <v>87</v>
       </c>
     </row>
@@ -2076,7 +2097,7 @@
       <c r="B90" s="1" t="s">
         <v>162</v>
       </c>
-      <c r="C90" s="3" t="s">
+      <c r="C90" s="2" t="s">
         <v>163</v>
       </c>
     </row>
@@ -2087,7 +2108,7 @@
       <c r="B91" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="C91" s="3" t="s">
+      <c r="C91" s="2" t="s">
         <v>33</v>
       </c>
     </row>
@@ -2098,7 +2119,7 @@
       <c r="B92" s="1" t="s">
         <v>166</v>
       </c>
-      <c r="C92" s="3" t="s">
+      <c r="C92" s="2" t="s">
         <v>167</v>
       </c>
     </row>
@@ -2109,7 +2130,7 @@
       <c r="B93" s="1" t="s">
         <v>169</v>
       </c>
-      <c r="C93" s="3" t="s">
+      <c r="C93" s="2" t="s">
         <v>170</v>
       </c>
     </row>
@@ -2128,101 +2149,131 @@
       <c r="B95" s="1" t="s">
         <v>174</v>
       </c>
-      <c r="C95" s="3" t="s">
+      <c r="C95" s="2" t="s">
         <v>175</v>
       </c>
     </row>
     <row r="96" ht="15">
-      <c r="A96" s="2" t="s">
+      <c r="A96" s="1" t="s">
         <v>176</v>
       </c>
-      <c r="B96" s="2" t="s">
+      <c r="B96" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="C96" s="3" t="s">
+      <c r="C96" s="2" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="97" ht="15">
-      <c r="A97" s="2" t="s">
+      <c r="A97" s="1" t="s">
         <v>177</v>
       </c>
-      <c r="B97" s="2" t="s">
+      <c r="B97" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="C97" s="4" t="s">
+      <c r="C97" s="3" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="98" ht="15">
-      <c r="A98" s="2" t="s">
+      <c r="A98" s="1" t="s">
         <v>178</v>
       </c>
-      <c r="B98" s="2" t="s">
+      <c r="B98" s="1" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="99" ht="15">
-      <c r="A99" s="2" t="s">
+      <c r="A99" s="1" t="s">
         <v>179</v>
       </c>
-      <c r="B99" s="2" t="s">
+      <c r="B99" s="1" t="s">
         <v>180</v>
       </c>
-      <c r="C99" s="4" t="s">
+      <c r="C99" s="3" t="s">
         <v>181</v>
       </c>
     </row>
     <row r="100" ht="15">
-      <c r="A100" s="2" t="s">
+      <c r="A100" s="1" t="s">
         <v>182</v>
       </c>
-      <c r="B100" s="2" t="s">
+      <c r="B100" s="1" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="101" ht="15">
-      <c r="A101" s="2" t="s">
+      <c r="A101" s="1" t="s">
         <v>183</v>
       </c>
-      <c r="B101" s="2" t="s">
+      <c r="B101" s="1" t="s">
         <v>110</v>
       </c>
-      <c r="C101" s="3" t="s">
+      <c r="C101" s="2" t="s">
         <v>111</v>
       </c>
     </row>
     <row r="102" ht="15">
-      <c r="A102" s="2" t="s">
+      <c r="A102" s="1" t="s">
         <v>184</v>
       </c>
-      <c r="B102" s="2" t="s">
+      <c r="B102" s="1" t="s">
         <v>149</v>
       </c>
-      <c r="C102" s="3" t="s">
+      <c r="C102" s="2" t="s">
         <v>150</v>
       </c>
     </row>
     <row r="103" ht="15">
-      <c r="A103" s="2" t="s">
+      <c r="A103" s="1" t="s">
         <v>185</v>
       </c>
-      <c r="B103" s="2" t="s">
+      <c r="B103" s="1" t="s">
         <v>110</v>
       </c>
-      <c r="C103" s="3" t="s">
+      <c r="C103" s="2" t="s">
         <v>111</v>
       </c>
     </row>
     <row r="104" ht="15">
-      <c r="A104" s="2" t="s">
+      <c r="A104" s="1" t="s">
         <v>186</v>
       </c>
-      <c r="B104" s="2" t="s">
+      <c r="B104" s="1" t="s">
         <v>187</v>
       </c>
-      <c r="C104" s="4" t="s">
+      <c r="C104" s="3" t="s">
         <v>188</v>
+      </c>
+    </row>
+    <row r="105" ht="15">
+      <c r="A105" s="4" t="s">
+        <v>189</v>
+      </c>
+      <c r="B105" s="4" t="s">
+        <v>190</v>
+      </c>
+      <c r="C105" s="3" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="106" ht="15">
+      <c r="A106" s="4" t="s">
+        <v>192</v>
+      </c>
+      <c r="B106" s="4" t="s">
+        <v>193</v>
+      </c>
+      <c r="C106" s="3" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="107" ht="15">
+      <c r="A107" s="4" t="s">
+        <v>195</v>
+      </c>
+      <c r="B107" s="4" t="s">
+        <v>4</v>
       </c>
     </row>
   </sheetData>
@@ -2325,6 +2376,8 @@
     <hyperlink r:id="rId32" ref="C102"/>
     <hyperlink r:id="rId24" ref="C103"/>
     <hyperlink r:id="rId40" ref="C104"/>
+    <hyperlink r:id="rId41" ref="C105"/>
+    <hyperlink r:id="rId42" ref="C106"/>
   </hyperlinks>
   <printOptions headings="0" gridLines="0" horizontalCentered="0" verticalCentered="0"/>
   <pageMargins left="0.78750000000000009" right="0.78750000000000009" top="1.05277777777778" bottom="1.05277777777778" header="0.78750000000000009" footer="0.78750000000000009"/>

</xml_diff>

<commit_message>
fix: add new attendees to spreadsheet
</commit_message>
<xml_diff>
--- a/data/wg_attendees.xlsx
+++ b/data/wg_attendees.xlsx
@@ -1,23 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <workbookPr date1904="0"/>
-  <workbookProtection/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
+  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <bookViews>
     <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet sheetId="1" name="Sheet1" state="visible" r:id="rId4"/>
   </sheets>
-  <calcPr refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.001"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{D0CA8CA8-9F24-4464-BF8E-62219DCF47F9}"/>
-  </extLst>
+  <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="196" uniqueCount="196">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="324" uniqueCount="202">
   <si>
     <t>name</t>
   </si>
@@ -28,13 +25,13 @@
     <t>affiliation_url</t>
   </si>
   <si>
-    <t xml:space="preserve">Joseph Rickert</t>
+    <t>Joseph Rickert</t>
   </si>
   <si>
     <t>Unknown</t>
   </si>
   <si>
-    <t xml:space="preserve">Adrian Waddell</t>
+    <t>Adrian Waddell</t>
   </si>
   <si>
     <t>Roche/Genentech</t>
@@ -43,13 +40,13 @@
     <t>https://www.gene.com</t>
   </si>
   <si>
-    <t xml:space="preserve">Doug Kelkhoff</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tadeusz Lewandowski</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ning Leng</t>
+    <t>Doug Kelkhoff</t>
+  </si>
+  <si>
+    <t>Tadeusz Lewandowski</t>
+  </si>
+  <si>
+    <t>Ning Leng</t>
   </si>
   <si>
     <t>AbbVie</t>
@@ -58,13 +55,13 @@
     <t>https://www.abbvie.com/</t>
   </si>
   <si>
-    <t xml:space="preserve">Heng Wang</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Beverly Chin</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bob Engle</t>
+    <t>Heng Wang</t>
+  </si>
+  <si>
+    <t>Beverly Chin</t>
+  </si>
+  <si>
+    <t>Bob Engle</t>
   </si>
   <si>
     <t>Biogen</t>
@@ -73,25 +70,25 @@
     <t xml:space="preserve">https://www.biogen.com/en_us/home.html </t>
   </si>
   <si>
-    <t xml:space="preserve">Christopher Kania</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Nate Mockler</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tim Powell</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Juliane Manitz</t>
-  </si>
-  <si>
-    <t xml:space="preserve">EMD Serono</t>
+    <t>Christopher Kania</t>
+  </si>
+  <si>
+    <t>Nate Mockler</t>
+  </si>
+  <si>
+    <t>Tim Powell</t>
+  </si>
+  <si>
+    <t>Juliane Manitz</t>
+  </si>
+  <si>
+    <t>EMD Serono</t>
   </si>
   <si>
     <t xml:space="preserve">https://www.emdserono.com/us-en </t>
   </si>
   <si>
-    <t xml:space="preserve">Lyn Taylor</t>
+    <t>Lyn Taylor</t>
   </si>
   <si>
     <t>Phastar</t>
@@ -100,7 +97,7 @@
     <t>https://phastar.com/</t>
   </si>
   <si>
-    <t xml:space="preserve">Mike Stackhouse</t>
+    <t>Mike Stackhouse</t>
   </si>
   <si>
     <t>Atorus</t>
@@ -109,10 +106,10 @@
     <t xml:space="preserve">https://www.atorusresearch.com/ </t>
   </si>
   <si>
-    <t xml:space="preserve">Eli Miller</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Paul Schuette</t>
+    <t>Eli Miller</t>
+  </si>
+  <si>
+    <t>Paul Schuette</t>
   </si>
   <si>
     <t>FDA</t>
@@ -121,28 +118,28 @@
     <t>https://www.fda.gov/</t>
   </si>
   <si>
-    <t xml:space="preserve">Ethan Chen</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bryant Chen</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Jiang Xu</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Jizu Zhi</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Kevin Snyder</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hye Soo Cho</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Maria Matilde Kam</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sascha Ahrweiler</t>
+    <t>Ethan Chen</t>
+  </si>
+  <si>
+    <t>Bryant Chen</t>
+  </si>
+  <si>
+    <t>Jiang Xu</t>
+  </si>
+  <si>
+    <t>Jizu Zhi</t>
+  </si>
+  <si>
+    <t>Kevin Snyder</t>
+  </si>
+  <si>
+    <t>Hye Soo Cho</t>
+  </si>
+  <si>
+    <t>Maria Matilde Kam</t>
+  </si>
+  <si>
+    <t>Sascha Ahrweiler</t>
   </si>
   <si>
     <t>Bayer</t>
@@ -151,7 +148,7 @@
     <t>https://www.bayer.com/en/</t>
   </si>
   <si>
-    <t xml:space="preserve">Phil Bowsher</t>
+    <t>Phil Bowsher</t>
   </si>
   <si>
     <t>Posit</t>
@@ -160,7 +157,7 @@
     <t xml:space="preserve">https://posit.co </t>
   </si>
   <si>
-    <t xml:space="preserve">Yilong Zhang</t>
+    <t>Yilong Zhang</t>
   </si>
   <si>
     <t>Meta</t>
@@ -169,7 +166,7 @@
     <t xml:space="preserve">https://facebook.com </t>
   </si>
   <si>
-    <t xml:space="preserve">Keaven Anderson</t>
+    <t>Keaven Anderson</t>
   </si>
   <si>
     <t>Merck</t>
@@ -178,10 +175,10 @@
     <t xml:space="preserve">https://www.merck.com </t>
   </si>
   <si>
-    <t xml:space="preserve">Nan Xiao</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Gregory Chen</t>
+    <t>Nan Xiao</t>
+  </si>
+  <si>
+    <t>Gregory Chen</t>
   </si>
   <si>
     <t>MSD</t>
@@ -190,13 +187,13 @@
     <t xml:space="preserve">https://www.msd.com/ </t>
   </si>
   <si>
-    <t xml:space="preserve">Miriam Fossati</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Peikun Wu</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Paulo Bargo</t>
+    <t>Miriam Fossati</t>
+  </si>
+  <si>
+    <t>Peikun Wu</t>
+  </si>
+  <si>
+    <t>Paulo Bargo</t>
   </si>
   <si>
     <t>Janssen</t>
@@ -205,7 +202,7 @@
     <t>https://www.jnjmedtech.com</t>
   </si>
   <si>
-    <t xml:space="preserve">Andy Nicholls</t>
+    <t>Andy Nicholls</t>
   </si>
   <si>
     <t>GSK</t>
@@ -214,16 +211,16 @@
     <t xml:space="preserve">https://www.gsk.com/en-gb/home/ </t>
   </si>
   <si>
-    <t xml:space="preserve">Ojesh Upandhyay</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ellis Hughes</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ben Straub</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Kevin Bolger</t>
+    <t>Ojesh Upandhyay</t>
+  </si>
+  <si>
+    <t>Ellis Hughes</t>
+  </si>
+  <si>
+    <t>Ben Straub</t>
+  </si>
+  <si>
+    <t>Kevin Bolger</t>
   </si>
   <si>
     <t>Procogia</t>
@@ -232,16 +229,16 @@
     <t xml:space="preserve">https://procogia.com </t>
   </si>
   <si>
-    <t xml:space="preserve">Eric Nantz</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Eli Lilly</t>
+    <t>Eric Nantz</t>
+  </si>
+  <si>
+    <t>Eli Lilly</t>
   </si>
   <si>
     <t xml:space="preserve">https://lilly.com </t>
   </si>
   <si>
-    <t xml:space="preserve">Bella Feng</t>
+    <t>Bella Feng</t>
   </si>
   <si>
     <t>EQRx</t>
@@ -250,22 +247,22 @@
     <t xml:space="preserve">https://www.eqrx.com </t>
   </si>
   <si>
-    <t xml:space="preserve">Steven Hasendinckx</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Johnson &amp; Johnson</t>
+    <t>Steven Hasendinckx</t>
+  </si>
+  <si>
+    <t>Johnson &amp; Johnson</t>
   </si>
   <si>
     <t>https://www.jnj.com</t>
   </si>
   <si>
-    <t xml:space="preserve">Heidi Curinckx</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Renping Zhang</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hong Yan</t>
+    <t>Heidi Curinckx</t>
+  </si>
+  <si>
+    <t>Renping Zhang</t>
+  </si>
+  <si>
+    <t>Hong Yan</t>
   </si>
   <si>
     <t>Regeneron</t>
@@ -274,16 +271,16 @@
     <t xml:space="preserve">https://www.regeneron.com </t>
   </si>
   <si>
-    <t xml:space="preserve">Ari Siggaard Knoph</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Novo Nordisk</t>
+    <t>Ari Siggaard Knoph</t>
+  </si>
+  <si>
+    <t>Novo Nordisk</t>
   </si>
   <si>
     <t xml:space="preserve">https://www.novonordisk.com/ </t>
   </si>
   <si>
-    <t xml:space="preserve">Michael Blanks</t>
+    <t>Michael Blanks</t>
   </si>
   <si>
     <t>BeiGene</t>
@@ -292,28 +289,28 @@
     <t xml:space="preserve">https://www.beigene.com/ </t>
   </si>
   <si>
-    <t xml:space="preserve">Robert Devine</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ryan Johnson</t>
+    <t>Robert Devine</t>
+  </si>
+  <si>
+    <t>Ryan Johnson</t>
   </si>
   <si>
     <t xml:space="preserve">https://posit.co  </t>
   </si>
   <si>
-    <t xml:space="preserve">Emily Nguyan</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Frederic Saad</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Jonathan Tisack</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hao Wang</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Graeme Hickey</t>
+    <t>Emily Nguyan</t>
+  </si>
+  <si>
+    <t>Frederic Saad</t>
+  </si>
+  <si>
+    <t>Jonathan Tisack</t>
+  </si>
+  <si>
+    <t>Hao Wang</t>
+  </si>
+  <si>
+    <t>Graeme Hickey</t>
   </si>
   <si>
     <t>Metronic</t>
@@ -322,19 +319,19 @@
     <t xml:space="preserve">https://www.medtronic.com/us-en/index.html </t>
   </si>
   <si>
-    <t xml:space="preserve">Michael Mayer</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Xin Qiu</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Shannon Lewis</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Joel Laxamana</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Stephanie Lussier</t>
+    <t>Michael Mayer</t>
+  </si>
+  <si>
+    <t>Xin Qiu</t>
+  </si>
+  <si>
+    <t>Shannon Lewis</t>
+  </si>
+  <si>
+    <t>Joel Laxamana</t>
+  </si>
+  <si>
+    <t>Stephanie Lussier</t>
   </si>
   <si>
     <t>Moderna</t>
@@ -343,10 +340,10 @@
     <t xml:space="preserve">https://www.modernatx.com </t>
   </si>
   <si>
-    <t xml:space="preserve">Thomas Neitmann</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sam Parmar</t>
+    <t>Thomas Neitmann</t>
+  </si>
+  <si>
+    <t>Sam Parmar</t>
   </si>
   <si>
     <t>Pfizer</t>
@@ -355,10 +352,10 @@
     <t xml:space="preserve">https://www.pfizer.com/ </t>
   </si>
   <si>
-    <t xml:space="preserve">Brian Sucher</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dadong Zhang</t>
+    <t>Brian Sucher</t>
+  </si>
+  <si>
+    <t>Dadong Zhang</t>
   </si>
   <si>
     <t>Illumina</t>
@@ -367,16 +364,16 @@
     <t xml:space="preserve">https://www.illumina.com/ </t>
   </si>
   <si>
-    <t xml:space="preserve">Yutong Liu</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lei Zhao</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Honghong Zhou</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Saghir Bashir</t>
+    <t>Yutong Liu</t>
+  </si>
+  <si>
+    <t>Lei Zhao</t>
+  </si>
+  <si>
+    <t>Honghong Zhou</t>
+  </si>
+  <si>
+    <t>Saghir Bashir</t>
   </si>
   <si>
     <t>Argenx</t>
@@ -385,109 +382,109 @@
     <t xml:space="preserve">https://www.argenx.com/ </t>
   </si>
   <si>
-    <t xml:space="preserve">Sean Healey</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Gabriel Becker</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Rupam Bhattacharyya</t>
-  </si>
-  <si>
-    <t xml:space="preserve">University of Michigan</t>
+    <t>Sean Healey</t>
+  </si>
+  <si>
+    <t>Gabriel Becker</t>
+  </si>
+  <si>
+    <t>Rupam Bhattacharyya</t>
+  </si>
+  <si>
+    <t>University of Michigan</t>
   </si>
   <si>
     <t xml:space="preserve">https://publichealth.umich.edu/ </t>
   </si>
   <si>
-    <t xml:space="preserve">Helena Sviglin</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Neetu Sangari</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Phanikumar Tata</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Syneos Health</t>
+    <t>Helena Sviglin</t>
+  </si>
+  <si>
+    <t>Neetu Sangari</t>
+  </si>
+  <si>
+    <t>Phanikumar Tata</t>
+  </si>
+  <si>
+    <t>Syneos Health</t>
   </si>
   <si>
     <t xml:space="preserve">https://www.syneoshealth.com/ </t>
   </si>
   <si>
-    <t xml:space="preserve">Kui Schen</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Estella Dong</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Yiwen Luo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bryan Tegomoh</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CDC Foundation</t>
+    <t>Kui Schen</t>
+  </si>
+  <si>
+    <t>Estella Dong</t>
+  </si>
+  <si>
+    <t>Yiwen Luo</t>
+  </si>
+  <si>
+    <t>Bryan Tegomoh</t>
+  </si>
+  <si>
+    <t>CDC Foundation</t>
   </si>
   <si>
     <t xml:space="preserve">https://www.cdcfoundation.org/ </t>
   </si>
   <si>
-    <t xml:space="preserve">Coline Zeballos</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Luke Schantz</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R Consortium</t>
+    <t>Coline Zeballos</t>
+  </si>
+  <si>
+    <t>Luke Schantz</t>
+  </si>
+  <si>
+    <t>R Consortium</t>
   </si>
   <si>
     <t>https://www.r-consortium.org</t>
   </si>
   <si>
-    <t xml:space="preserve">Andrew Borgman</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bristol Myers Squibb</t>
+    <t>Andrew Borgman</t>
+  </si>
+  <si>
+    <t>Bristol Myers Squibb</t>
   </si>
   <si>
     <t xml:space="preserve">https://www.bms.com/ </t>
   </si>
   <si>
-    <t xml:space="preserve">Henry Wang</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Chenguang Wang</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Qin Lin</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Kevin Kunzmann</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Boehringer Ingelheim</t>
+    <t>Henry Wang</t>
+  </si>
+  <si>
+    <t>Chenguang Wang</t>
+  </si>
+  <si>
+    <t>Qin Lin</t>
+  </si>
+  <si>
+    <t>Kevin Kunzmann</t>
+  </si>
+  <si>
+    <t>Boehringer Ingelheim</t>
   </si>
   <si>
     <t xml:space="preserve">https://www.boehringer-ingelheim.com/ </t>
   </si>
   <si>
-    <t xml:space="preserve">Michael Kane</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MD Anderson Cancer Institute</t>
+    <t>Michael Kane</t>
+  </si>
+  <si>
+    <t>MD Anderson Cancer Institute</t>
   </si>
   <si>
     <t xml:space="preserve">https://www.mdanderson.org/ </t>
   </si>
   <si>
-    <t xml:space="preserve">Terry Christiani</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Amanda Martin</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Andre Couturier</t>
+    <t>Terry Christiani</t>
+  </si>
+  <si>
+    <t>Amanda Martin</t>
+  </si>
+  <si>
+    <t>Andre Couturier</t>
   </si>
   <si>
     <t>Sanofi</t>
@@ -496,13 +493,13 @@
     <t xml:space="preserve">https://www.sanofi.com/ </t>
   </si>
   <si>
-    <t xml:space="preserve">Nicholas Masel</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lovemore Gakava</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Katie Harding</t>
+    <t>Nicholas Masel</t>
+  </si>
+  <si>
+    <t>Lovemore Gakava</t>
+  </si>
+  <si>
+    <t>Katie Harding</t>
   </si>
   <si>
     <t>Freenome</t>
@@ -511,10 +508,10 @@
     <t xml:space="preserve">https://www.freenome.com/ </t>
   </si>
   <si>
-    <t xml:space="preserve">Youn Kyeong Chang</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sam Hume</t>
+    <t>Youn Kyeong Chang</t>
+  </si>
+  <si>
+    <t>Sam Hume</t>
   </si>
   <si>
     <t>CDISC</t>
@@ -523,7 +520,7 @@
     <t xml:space="preserve">https://www.cdisc.org/ </t>
   </si>
   <si>
-    <t xml:space="preserve">Camille Calmasini</t>
+    <t>Camille Calmasini</t>
   </si>
   <si>
     <t>Natera</t>
@@ -532,52 +529,55 @@
     <t>https://www.natera.com/</t>
   </si>
   <si>
-    <t xml:space="preserve">Jim Rothstein</t>
+    <t>Jim Rothstein</t>
   </si>
   <si>
     <t>Freelance</t>
   </si>
   <si>
-    <t xml:space="preserve">Nabil Baugher</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Baseline AI</t>
+    <t>Nabil Baugher</t>
+  </si>
+  <si>
+    <t>Baseline AI</t>
   </si>
   <si>
     <t>https://www.baselinetrials.com</t>
   </si>
   <si>
-    <t xml:space="preserve">Gabriel Krotkov</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hong Zheng</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Karthik Velega</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Luis Osorio</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Los Angeles Count Department of Public Health</t>
+    <t>Gabriel Krotkov</t>
+  </si>
+  <si>
+    <t>Hong Zheng</t>
+  </si>
+  <si>
+    <t>Karthik Velega</t>
+  </si>
+  <si>
+    <t>Luis Osorio</t>
+  </si>
+  <si>
+    <t>Los Angeles Count Department of Public Health</t>
   </si>
   <si>
     <t>http://publichealth.lacounty.gov/</t>
   </si>
   <si>
-    <t xml:space="preserve">Sara Z</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sydney Dennison</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Vital Reddy Jaggavarapu</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Yogesh Gupta</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Jared Woolfolk</t>
+    <t>Sarah Zanzoul</t>
+  </si>
+  <si>
+    <t>https://www.pfizer.com/</t>
+  </si>
+  <si>
+    <t>Sydney Dennison</t>
+  </si>
+  <si>
+    <t>Vital Reddy Jaggavarapu</t>
+  </si>
+  <si>
+    <t>Yogesh Gupta</t>
+  </si>
+  <si>
+    <t>Jared Woolfolk</t>
   </si>
   <si>
     <t>Cytel</t>
@@ -586,50 +586,68 @@
     <t>https://cytel.com/</t>
   </si>
   <si>
-    <t xml:space="preserve">Vinod Kumar</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TruMines Clinical</t>
+    <t>Vinod Kumar</t>
+  </si>
+  <si>
+    <t>TruMines Clinical</t>
   </si>
   <si>
     <t>https://trumindsclinical.com/</t>
   </si>
   <si>
-    <t xml:space="preserve">Chi-Hua Huang</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Astellas Pharmaceuticals</t>
+    <t>Chi-Hua Huang</t>
+  </si>
+  <si>
+    <t>Astellas Pharmaceuticals</t>
   </si>
   <si>
     <t>https://www.astellas.com/en/</t>
   </si>
   <si>
     <t>Ram</t>
+  </si>
+  <si>
+    <t>Brandon Sucher</t>
+  </si>
+  <si>
+    <t>https://www.modernatx.com/</t>
+  </si>
+  <si>
+    <t>Dmitry Kolosov</t>
+  </si>
+  <si>
+    <t>Vital Jaggavarapu</t>
+  </si>
+  <si>
+    <t>https://www.boehringer-ingelheim.com/</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="4">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
-      <sz val="10.000000"/>
       <color theme="1"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <color theme="1"/>
+      <sz val="10"/>
       <name val="Arial"/>
     </font>
     <font>
-      <sz val="10.000000"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10.000000"/>
       <color indexed="4"/>
+      <sz val="10"/>
       <name val="Arial"/>
     </font>
     <font>
       <u/>
-      <sz val="10.000000"/>
       <color theme="10"/>
+      <sz val="10"/>
       <name val="Arial"/>
     </font>
   </fonts>
@@ -641,7 +659,14 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
     <border>
       <left style="none"/>
       <right style="none"/>
@@ -650,46 +675,26 @@
       <diagonal style="none"/>
     </border>
   </borders>
-  <cellStyleXfs count="6">
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
-      <protection hidden="0" locked="1"/>
-    </xf>
-    <xf fontId="1" fillId="0" borderId="0" numFmtId="43" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyProtection="0"/>
-    <xf fontId="1" fillId="0" borderId="0" numFmtId="41" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyProtection="0"/>
-    <xf fontId="1" fillId="0" borderId="0" numFmtId="44" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyProtection="0"/>
-    <xf fontId="1" fillId="0" borderId="0" numFmtId="42" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyProtection="0"/>
-    <xf fontId="1" fillId="0" borderId="0" numFmtId="9" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyProtection="0"/>
+  <cellStyleXfs count="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyProtection="0">
-      <protection hidden="0" locked="1"/>
-    </xf>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyProtection="1">
-      <protection hidden="0" locked="1"/>
-    </xf>
-    <xf fontId="2" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyProtection="1">
-      <protection hidden="0" locked="1"/>
-    </xf>
-    <xf fontId="3" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyProtection="1">
-      <protection hidden="0" locked="1"/>
-    </xf>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyProtection="1">
-      <protection hidden="0" locked="1"/>
-    </xf>
+  <cellXfs count="4">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
-  <cellStyles count="6">
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Comma" xfId="1" builtinId="3"/>
-    <cellStyle name="Comma [0]" xfId="2" builtinId="6"/>
-    <cellStyle name="Currency" xfId="3" builtinId="4"/>
-    <cellStyle name="Currency [0]" xfId="4" builtinId="7"/>
-    <cellStyle name="Percent" xfId="5" builtinId="5"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
@@ -1104,19 +1109,19 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
-  <sheetPr filterMode="0">
-    <outlinePr applyStyles="0" summaryBelow="1" summaryRight="1" showOutlineSymbols="1"/>
-    <pageSetUpPr autoPageBreaks="1" fitToPage="0"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <sheetFormatPr defaultColWidth="11.60546875" defaultRowHeight="15"/>
+  <dimension ref="A1:C110"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="11.60546875"/>
   <cols>
-    <col customWidth="1" min="1" max="1" style="1" width="28.109999999999999"/>
-    <col customWidth="1" min="2" max="2" style="1" width="38.50390625"/>
-    <col customWidth="1" min="3" max="3" style="1" width="36.299999999999997"/>
+    <col min="1" max="1" width="28.11" style="1" customWidth="1"/>
+    <col min="2" max="2" width="38.50390625" style="1" customWidth="1"/>
+    <col min="3" max="3" width="36.3" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="12.800000000000001">
+    <row r="1" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1127,7 +1132,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" ht="12.800000000000001">
+    <row r="2" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>3</v>
       </c>
@@ -1136,7 +1141,7 @@
       </c>
       <c r="C2" s="2"/>
     </row>
-    <row r="3" ht="12.800000000000001">
+    <row r="3" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>5</v>
       </c>
@@ -1147,7 +1152,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="4" ht="12.800000000000001">
+    <row r="4" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>8</v>
       </c>
@@ -1158,7 +1163,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="5" ht="12.800000000000001">
+    <row r="5" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>9</v>
       </c>
@@ -1169,7 +1174,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="6" ht="12.800000000000001">
+    <row r="6" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>10</v>
       </c>
@@ -1180,7 +1185,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="7" ht="12.800000000000001">
+    <row r="7" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>13</v>
       </c>
@@ -1191,7 +1196,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="8" ht="12.800000000000001">
+    <row r="8" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>14</v>
       </c>
@@ -1202,7 +1207,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="9" ht="12.800000000000001">
+    <row r="9" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>15</v>
       </c>
@@ -1213,7 +1218,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="10" ht="12.800000000000001">
+    <row r="10" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>18</v>
       </c>
@@ -1224,7 +1229,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="11" ht="12.800000000000001">
+    <row r="11" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>19</v>
       </c>
@@ -1235,7 +1240,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="12" ht="12.800000000000001">
+    <row r="12" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>20</v>
       </c>
@@ -1246,7 +1251,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="13" ht="12.800000000000001">
+    <row r="13" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
         <v>21</v>
       </c>
@@ -1257,7 +1262,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="14" ht="12.800000000000001">
+    <row r="14" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
         <v>24</v>
       </c>
@@ -1268,7 +1273,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="15" ht="12.800000000000001">
+    <row r="15" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
         <v>27</v>
       </c>
@@ -1279,7 +1284,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="16" ht="12.800000000000001">
+    <row r="16" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
         <v>30</v>
       </c>
@@ -1290,7 +1295,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="17" ht="12.800000000000001">
+    <row r="17" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
         <v>31</v>
       </c>
@@ -1301,7 +1306,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="18" ht="12.800000000000001">
+    <row r="18" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
         <v>34</v>
       </c>
@@ -1312,7 +1317,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="19" ht="12.800000000000001">
+    <row r="19" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
         <v>35</v>
       </c>
@@ -1323,7 +1328,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="20" ht="12.800000000000001">
+    <row r="20" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
         <v>36</v>
       </c>
@@ -1334,7 +1339,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="21" ht="12.800000000000001">
+    <row r="21" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
         <v>37</v>
       </c>
@@ -1345,7 +1350,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="22" ht="12.800000000000001">
+    <row r="22" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
         <v>38</v>
       </c>
@@ -1356,7 +1361,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="23" ht="12.800000000000001">
+    <row r="23" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
         <v>39</v>
       </c>
@@ -1367,7 +1372,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="24" ht="12.800000000000001">
+    <row r="24" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
         <v>40</v>
       </c>
@@ -1378,7 +1383,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="25" ht="12.800000000000001">
+    <row r="25" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
         <v>41</v>
       </c>
@@ -1389,7 +1394,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="26" ht="12.800000000000001">
+    <row r="26" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
         <v>44</v>
       </c>
@@ -1400,7 +1405,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="27" ht="12.800000000000001">
+    <row r="27" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
         <v>47</v>
       </c>
@@ -1411,7 +1416,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="28" ht="12.800000000000001">
+    <row r="28" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
         <v>50</v>
       </c>
@@ -1422,7 +1427,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="29" ht="12.800000000000001">
+    <row r="29" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" s="1" t="s">
         <v>53</v>
       </c>
@@ -1433,7 +1438,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="30" ht="12.800000000000001">
+    <row r="30" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30" s="1" t="s">
         <v>54</v>
       </c>
@@ -1444,7 +1449,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="31" ht="12.800000000000001">
+    <row r="31" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A31" s="1" t="s">
         <v>57</v>
       </c>
@@ -1455,7 +1460,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="32" ht="12.800000000000001">
+    <row r="32" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A32" s="1" t="s">
         <v>58</v>
       </c>
@@ -1466,7 +1471,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="33" ht="12.800000000000001">
+    <row r="33" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A33" s="1" t="s">
         <v>59</v>
       </c>
@@ -1477,7 +1482,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="34" ht="12.800000000000001">
+    <row r="34" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A34" s="1" t="s">
         <v>62</v>
       </c>
@@ -1488,7 +1493,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="35" ht="12.800000000000001">
+    <row r="35" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A35" s="1" t="s">
         <v>65</v>
       </c>
@@ -1499,7 +1504,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="36" ht="12.800000000000001">
+    <row r="36" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A36" s="1" t="s">
         <v>66</v>
       </c>
@@ -1510,7 +1515,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="37" ht="12.800000000000001">
+    <row r="37" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A37" s="1" t="s">
         <v>67</v>
       </c>
@@ -1521,7 +1526,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="38" ht="12.800000000000001">
+    <row r="38" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A38" s="1" t="s">
         <v>68</v>
       </c>
@@ -1532,7 +1537,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="39" ht="12.800000000000001">
+    <row r="39" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A39" s="1" t="s">
         <v>71</v>
       </c>
@@ -1543,7 +1548,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="40" ht="12.800000000000001">
+    <row r="40" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A40" s="1" t="s">
         <v>74</v>
       </c>
@@ -1554,7 +1559,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="41" ht="12.800000000000001">
+    <row r="41" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A41" s="1" t="s">
         <v>77</v>
       </c>
@@ -1565,7 +1570,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="42" ht="12.800000000000001">
+    <row r="42" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A42" s="1" t="s">
         <v>80</v>
       </c>
@@ -1576,7 +1581,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="43" ht="12.800000000000001">
+    <row r="43" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A43" s="1" t="s">
         <v>81</v>
       </c>
@@ -1587,7 +1592,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="44" ht="12.800000000000001">
+    <row r="44" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A44" s="1" t="s">
         <v>82</v>
       </c>
@@ -1598,7 +1603,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="45" ht="12.800000000000001">
+    <row r="45" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A45" s="1" t="s">
         <v>85</v>
       </c>
@@ -1609,7 +1614,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="46" ht="12.800000000000001">
+    <row r="46" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A46" s="1" t="s">
         <v>88</v>
       </c>
@@ -1620,7 +1625,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="47" ht="12.800000000000001">
+    <row r="47" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A47" s="1" t="s">
         <v>91</v>
       </c>
@@ -1631,7 +1636,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="48" ht="12.800000000000001">
+    <row r="48" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A48" s="1" t="s">
         <v>92</v>
       </c>
@@ -1642,7 +1647,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="49" ht="12.800000000000001">
+    <row r="49" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A49" s="1" t="s">
         <v>94</v>
       </c>
@@ -1653,7 +1658,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="50" ht="12.800000000000001">
+    <row r="50" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A50" s="1" t="s">
         <v>95</v>
       </c>
@@ -1664,7 +1669,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="51" ht="12.800000000000001">
+    <row r="51" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A51" s="1" t="s">
         <v>96</v>
       </c>
@@ -1675,7 +1680,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="52" ht="12.800000000000001">
+    <row r="52" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A52" s="1" t="s">
         <v>97</v>
       </c>
@@ -1686,7 +1691,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="53" ht="12.800000000000001">
+    <row r="53" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A53" s="1" t="s">
         <v>98</v>
       </c>
@@ -1697,7 +1702,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="54" ht="12.800000000000001">
+    <row r="54" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A54" s="1" t="s">
         <v>101</v>
       </c>
@@ -1708,7 +1713,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="55" ht="12.800000000000001">
+    <row r="55" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A55" s="1" t="s">
         <v>102</v>
       </c>
@@ -1719,7 +1724,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="56" ht="12.800000000000001">
+    <row r="56" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A56" s="1" t="s">
         <v>103</v>
       </c>
@@ -1730,7 +1735,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="57" ht="12.800000000000001">
+    <row r="57" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A57" s="1" t="s">
         <v>104</v>
       </c>
@@ -1741,7 +1746,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="58" ht="12.800000000000001">
+    <row r="58" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A58" s="1" t="s">
         <v>105</v>
       </c>
@@ -1752,7 +1757,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="59" ht="12.800000000000001">
+    <row r="59" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A59" s="1" t="s">
         <v>108</v>
       </c>
@@ -1763,7 +1768,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="60" ht="12.800000000000001">
+    <row r="60" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A60" s="1" t="s">
         <v>109</v>
       </c>
@@ -1774,7 +1779,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="61" ht="12.800000000000001">
+    <row r="61" ht="12.8" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A61" s="1" t="s">
         <v>112</v>
       </c>
@@ -1782,7 +1787,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="62" ht="12.800000000000001">
+    <row r="62" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A62" s="1" t="s">
         <v>113</v>
       </c>
@@ -1793,7 +1798,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="63" ht="12.800000000000001">
+    <row r="63" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A63" s="1" t="s">
         <v>116</v>
       </c>
@@ -1804,7 +1809,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="64" ht="12.800000000000001">
+    <row r="64" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A64" s="1" t="s">
         <v>117</v>
       </c>
@@ -1815,7 +1820,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="65" ht="12.800000000000001">
+    <row r="65" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A65" s="1" t="s">
         <v>118</v>
       </c>
@@ -1826,7 +1831,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="66" ht="12.800000000000001">
+    <row r="66" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A66" s="1" t="s">
         <v>119</v>
       </c>
@@ -1837,7 +1842,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="67" ht="12.800000000000001">
+    <row r="67" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A67" s="1" t="s">
         <v>122</v>
       </c>
@@ -1848,7 +1853,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="68" ht="12.800000000000001">
+    <row r="68" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A68" s="1" t="s">
         <v>123</v>
       </c>
@@ -1859,7 +1864,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="69" ht="12.800000000000001">
+    <row r="69" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A69" s="1" t="s">
         <v>124</v>
       </c>
@@ -1870,7 +1875,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="70" ht="12.800000000000001">
+    <row r="70" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A70" s="1" t="s">
         <v>127</v>
       </c>
@@ -1881,7 +1886,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="71" ht="12.800000000000001">
+    <row r="71" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A71" s="1" t="s">
         <v>128</v>
       </c>
@@ -1892,7 +1897,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="72" ht="12.800000000000001">
+    <row r="72" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A72" s="1" t="s">
         <v>129</v>
       </c>
@@ -1903,7 +1908,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="73" ht="12.800000000000001">
+    <row r="73" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A73" s="1" t="s">
         <v>132</v>
       </c>
@@ -1914,7 +1919,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="74" ht="12.800000000000001">
+    <row r="74" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A74" s="1" t="s">
         <v>133</v>
       </c>
@@ -1925,7 +1930,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="75" ht="12.800000000000001">
+    <row r="75" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A75" s="1" t="s">
         <v>134</v>
       </c>
@@ -1936,7 +1941,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="76" ht="12.800000000000001">
+    <row r="76" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A76" s="1" t="s">
         <v>135</v>
       </c>
@@ -1947,7 +1952,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="77" ht="12.800000000000001">
+    <row r="77" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A77" s="1" t="s">
         <v>138</v>
       </c>
@@ -1958,7 +1963,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="78" ht="12.800000000000001">
+    <row r="78" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A78" s="1" t="s">
         <v>139</v>
       </c>
@@ -1969,7 +1974,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="79" ht="12.800000000000001">
+    <row r="79" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A79" s="1" t="s">
         <v>142</v>
       </c>
@@ -1980,7 +1985,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="80" ht="12.800000000000001">
+    <row r="80" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A80" s="1" t="s">
         <v>145</v>
       </c>
@@ -1991,7 +1996,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="81" ht="12.800000000000001">
+    <row r="81" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A81" s="1" t="s">
         <v>146</v>
       </c>
@@ -2002,7 +2007,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="82" ht="12.800000000000001">
+    <row r="82" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A82" s="1" t="s">
         <v>147</v>
       </c>
@@ -2013,7 +2018,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="83" ht="12.800000000000001">
+    <row r="83" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A83" s="1" t="s">
         <v>148</v>
       </c>
@@ -2024,7 +2029,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="84" ht="12.800000000000001">
+    <row r="84" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A84" s="1" t="s">
         <v>151</v>
       </c>
@@ -2035,7 +2040,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="85" ht="12.800000000000001">
+    <row r="85" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A85" s="1" t="s">
         <v>154</v>
       </c>
@@ -2046,7 +2051,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="86" ht="12.800000000000001">
+    <row r="86" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A86" s="1" t="s">
         <v>155</v>
       </c>
@@ -2057,7 +2062,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="87" ht="12.800000000000001">
+    <row r="87" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A87" s="1" t="s">
         <v>156</v>
       </c>
@@ -2068,7 +2073,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="88" ht="12.800000000000001">
+    <row r="88" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A88" s="1" t="s">
         <v>159</v>
       </c>
@@ -2079,7 +2084,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="89" ht="12.800000000000001">
+    <row r="89" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A89" s="1" t="s">
         <v>160</v>
       </c>
@@ -2090,7 +2095,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="90" ht="12.800000000000001">
+    <row r="90" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A90" s="1" t="s">
         <v>161</v>
       </c>
@@ -2101,7 +2106,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="91" ht="12.800000000000001">
+    <row r="91" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A91" s="1" t="s">
         <v>164</v>
       </c>
@@ -2112,7 +2117,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="92" ht="12.800000000000001">
+    <row r="92" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A92" s="1" t="s">
         <v>165</v>
       </c>
@@ -2123,7 +2128,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="93" ht="12.800000000000001">
+    <row r="93" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A93" s="1" t="s">
         <v>168</v>
       </c>
@@ -2134,7 +2139,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="94" ht="12.800000000000001">
+    <row r="94" ht="12.8" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A94" s="1" t="s">
         <v>171</v>
       </c>
@@ -2142,7 +2147,7 @@
         <v>172</v>
       </c>
     </row>
-    <row r="95" ht="12.800000000000001">
+    <row r="95" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A95" s="1" t="s">
         <v>173</v>
       </c>
@@ -2153,7 +2158,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="96" ht="15">
+    <row r="96" ht="15" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A96" s="1" t="s">
         <v>176</v>
       </c>
@@ -2164,7 +2169,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="97" ht="15">
+    <row r="97" ht="15" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A97" s="1" t="s">
         <v>177</v>
       </c>
@@ -2175,7 +2180,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="98" ht="15">
+    <row r="98" ht="15" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A98" s="1" t="s">
         <v>178</v>
       </c>
@@ -2183,7 +2188,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="99" ht="15">
+    <row r="99" ht="15" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A99" s="1" t="s">
         <v>179</v>
       </c>
@@ -2194,17 +2199,20 @@
         <v>181</v>
       </c>
     </row>
-    <row r="100" ht="15">
+    <row r="100" ht="15" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A100" s="1" t="s">
         <v>182</v>
       </c>
       <c r="B100" s="1" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="101" ht="15">
+        <v>110</v>
+      </c>
+      <c r="C100" s="1" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="101" ht="15" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A101" s="1" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="B101" s="1" t="s">
         <v>110</v>
@@ -2213,9 +2221,9 @@
         <v>111</v>
       </c>
     </row>
-    <row r="102" ht="15">
+    <row r="102" ht="15" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A102" s="1" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="B102" s="1" t="s">
         <v>149</v>
@@ -2224,9 +2232,9 @@
         <v>150</v>
       </c>
     </row>
-    <row r="103" ht="15">
+    <row r="103" ht="15" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A103" s="1" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="B103" s="1" t="s">
         <v>110</v>
@@ -2235,153 +2243,182 @@
         <v>111</v>
       </c>
     </row>
-    <row r="104" ht="15">
+    <row r="104" ht="15" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A104" s="1" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="B104" s="1" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="C104" s="3" t="s">
-        <v>188</v>
-      </c>
-    </row>
-    <row r="105" ht="15">
-      <c r="A105" s="4" t="s">
         <v>189</v>
       </c>
-      <c r="B105" s="4" t="s">
+    </row>
+    <row r="105" ht="15" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A105" s="1" t="s">
         <v>190</v>
       </c>
+      <c r="B105" s="1" t="s">
+        <v>191</v>
+      </c>
       <c r="C105" s="3" t="s">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="106" ht="15">
-      <c r="A106" s="4" t="s">
         <v>192</v>
       </c>
-      <c r="B106" s="4" t="s">
+    </row>
+    <row r="106" ht="15" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A106" s="1" t="s">
         <v>193</v>
       </c>
+      <c r="B106" s="1" t="s">
+        <v>194</v>
+      </c>
       <c r="C106" s="3" t="s">
-        <v>194</v>
-      </c>
-    </row>
-    <row r="107" ht="15">
-      <c r="A107" s="4" t="s">
         <v>195</v>
       </c>
-      <c r="B107" s="4" t="s">
+    </row>
+    <row r="107" ht="15" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A107" s="1" t="s">
+        <v>196</v>
+      </c>
+      <c r="B107" s="1" t="s">
         <v>4</v>
+      </c>
+    </row>
+    <row r="108" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A108" s="1" t="s">
+        <v>197</v>
+      </c>
+      <c r="B108" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="C108" s="1" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="109" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A109" s="1" t="s">
+        <v>199</v>
+      </c>
+      <c r="B109" s="1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="110" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A110" s="1" t="s">
+        <v>200</v>
+      </c>
+      <c r="B110" s="1" t="s">
+        <v>149</v>
+      </c>
+      <c r="C110" s="1" t="s">
+        <v>201</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink r:id="rId1" ref="C3"/>
-    <hyperlink r:id="rId1" ref="C4"/>
-    <hyperlink r:id="rId1" ref="C5"/>
-    <hyperlink r:id="rId2" ref="C6"/>
-    <hyperlink r:id="rId1" ref="C7"/>
-    <hyperlink r:id="rId1" ref="C8"/>
-    <hyperlink r:id="rId3" ref="C9"/>
-    <hyperlink r:id="rId3" ref="C10"/>
-    <hyperlink r:id="rId3" ref="C11"/>
-    <hyperlink r:id="rId3" ref="C12"/>
-    <hyperlink r:id="rId4" ref="C13"/>
-    <hyperlink r:id="rId5" ref="C14"/>
-    <hyperlink r:id="rId6" ref="C15"/>
-    <hyperlink r:id="rId6" ref="C16"/>
-    <hyperlink r:id="rId7" ref="C17"/>
-    <hyperlink r:id="rId7" ref="C18"/>
-    <hyperlink r:id="rId7" ref="C19"/>
-    <hyperlink r:id="rId7" ref="C20"/>
-    <hyperlink r:id="rId7" ref="C21"/>
-    <hyperlink r:id="rId7" ref="C22"/>
-    <hyperlink r:id="rId7" ref="C23"/>
-    <hyperlink r:id="rId7" ref="C24"/>
-    <hyperlink r:id="rId8" ref="C25"/>
-    <hyperlink r:id="rId9" ref="C26"/>
-    <hyperlink r:id="rId10" ref="C27"/>
-    <hyperlink r:id="rId11" ref="C28"/>
-    <hyperlink r:id="rId11" ref="C29"/>
-    <hyperlink r:id="rId12" ref="C30"/>
-    <hyperlink r:id="rId11" ref="C31"/>
-    <hyperlink r:id="rId11" ref="C32"/>
-    <hyperlink r:id="rId13" ref="C33"/>
-    <hyperlink r:id="rId14" ref="C34"/>
-    <hyperlink r:id="rId14" ref="C35"/>
-    <hyperlink r:id="rId14" ref="C36"/>
-    <hyperlink r:id="rId14" ref="C37"/>
-    <hyperlink r:id="rId15" ref="C38"/>
-    <hyperlink r:id="rId16" ref="C39"/>
-    <hyperlink r:id="rId17" ref="C40"/>
-    <hyperlink r:id="rId18" ref="C41"/>
-    <hyperlink r:id="rId18" ref="C42"/>
-    <hyperlink r:id="rId18" ref="C43"/>
-    <hyperlink r:id="rId19" ref="C44"/>
-    <hyperlink r:id="rId20" ref="C45"/>
-    <hyperlink r:id="rId21" ref="C46"/>
-    <hyperlink r:id="rId18" ref="C47"/>
-    <hyperlink r:id="rId9" ref="C48"/>
-    <hyperlink r:id="rId7" ref="C49"/>
-    <hyperlink r:id="rId13" ref="C50"/>
-    <hyperlink r:id="rId21" ref="C51"/>
-    <hyperlink r:id="rId7" ref="C52"/>
-    <hyperlink r:id="rId22" ref="C53"/>
-    <hyperlink r:id="rId9" ref="C54"/>
-    <hyperlink r:id="rId18" ref="C55"/>
-    <hyperlink r:id="rId21" ref="C56"/>
-    <hyperlink r:id="rId1" ref="C57"/>
-    <hyperlink r:id="rId23" ref="C58"/>
-    <hyperlink r:id="rId1" ref="C59"/>
-    <hyperlink r:id="rId24" ref="C60"/>
-    <hyperlink r:id="rId25" ref="C62"/>
-    <hyperlink r:id="rId23" ref="C63"/>
-    <hyperlink r:id="rId1" ref="C64"/>
-    <hyperlink r:id="rId23" ref="C65"/>
-    <hyperlink r:id="rId26" ref="C66"/>
-    <hyperlink r:id="rId24" ref="C67"/>
-    <hyperlink r:id="rId1" ref="C68"/>
-    <hyperlink r:id="rId27" ref="C69"/>
-    <hyperlink r:id="rId7" ref="C70"/>
-    <hyperlink r:id="rId24" ref="C71"/>
-    <hyperlink r:id="rId28" ref="C72"/>
-    <hyperlink r:id="rId8" ref="C73"/>
-    <hyperlink r:id="rId8" ref="C74"/>
-    <hyperlink r:id="rId11" ref="C75"/>
-    <hyperlink r:id="rId29" ref="C76"/>
-    <hyperlink r:id="rId1" ref="C77"/>
-    <hyperlink r:id="rId30" ref="C78"/>
-    <hyperlink r:id="rId31" ref="C79"/>
-    <hyperlink r:id="rId1" ref="C80"/>
-    <hyperlink r:id="rId19" ref="C81"/>
-    <hyperlink r:id="rId14" ref="C82"/>
-    <hyperlink r:id="rId32" ref="C83"/>
-    <hyperlink r:id="rId33" ref="C84"/>
-    <hyperlink r:id="rId30" ref="C85"/>
-    <hyperlink r:id="rId30" ref="C86"/>
-    <hyperlink r:id="rId34" ref="C87"/>
-    <hyperlink r:id="rId18" ref="C88"/>
-    <hyperlink r:id="rId20" ref="C89"/>
-    <hyperlink r:id="rId35" ref="C90"/>
-    <hyperlink r:id="rId7" ref="C91"/>
-    <hyperlink r:id="rId36" ref="C92"/>
-    <hyperlink r:id="rId37" ref="C93"/>
-    <hyperlink r:id="rId38" ref="C95"/>
-    <hyperlink r:id="rId7" ref="C96"/>
-    <hyperlink r:id="rId8" ref="C97"/>
-    <hyperlink r:id="rId39" ref="C99"/>
-    <hyperlink r:id="rId24" ref="C101"/>
-    <hyperlink r:id="rId32" ref="C102"/>
-    <hyperlink r:id="rId24" ref="C103"/>
-    <hyperlink r:id="rId40" ref="C104"/>
-    <hyperlink r:id="rId41" ref="C105"/>
-    <hyperlink r:id="rId42" ref="C106"/>
+    <hyperlink ref="C3" r:id="rId1"/>
+    <hyperlink ref="C4" r:id="rId2"/>
+    <hyperlink ref="C5" r:id="rId3"/>
+    <hyperlink ref="C6" r:id="rId4"/>
+    <hyperlink ref="C7" r:id="rId5"/>
+    <hyperlink ref="C8" r:id="rId6"/>
+    <hyperlink ref="C9" r:id="rId7"/>
+    <hyperlink ref="C10" r:id="rId8"/>
+    <hyperlink ref="C11" r:id="rId9"/>
+    <hyperlink ref="C12" r:id="rId10"/>
+    <hyperlink ref="C13" r:id="rId11"/>
+    <hyperlink ref="C14" r:id="rId12"/>
+    <hyperlink ref="C15" r:id="rId13"/>
+    <hyperlink ref="C16" r:id="rId14"/>
+    <hyperlink ref="C17" r:id="rId15"/>
+    <hyperlink ref="C18" r:id="rId16"/>
+    <hyperlink ref="C19" r:id="rId17"/>
+    <hyperlink ref="C20" r:id="rId18"/>
+    <hyperlink ref="C21" r:id="rId19"/>
+    <hyperlink ref="C22" r:id="rId20"/>
+    <hyperlink ref="C23" r:id="rId21"/>
+    <hyperlink ref="C24" r:id="rId22"/>
+    <hyperlink ref="C25" r:id="rId23"/>
+    <hyperlink ref="C26" r:id="rId24"/>
+    <hyperlink ref="C27" r:id="rId25"/>
+    <hyperlink ref="C28" r:id="rId26"/>
+    <hyperlink ref="C29" r:id="rId27"/>
+    <hyperlink ref="C30" r:id="rId28"/>
+    <hyperlink ref="C31" r:id="rId29"/>
+    <hyperlink ref="C32" r:id="rId30"/>
+    <hyperlink ref="C33" r:id="rId31"/>
+    <hyperlink ref="C34" r:id="rId32"/>
+    <hyperlink ref="C35" r:id="rId33"/>
+    <hyperlink ref="C36" r:id="rId34"/>
+    <hyperlink ref="C37" r:id="rId35"/>
+    <hyperlink ref="C38" r:id="rId36"/>
+    <hyperlink ref="C39" r:id="rId37"/>
+    <hyperlink ref="C40" r:id="rId38"/>
+    <hyperlink ref="C41" r:id="rId39"/>
+    <hyperlink ref="C42" r:id="rId40"/>
+    <hyperlink ref="C43" r:id="rId41"/>
+    <hyperlink ref="C44" r:id="rId42"/>
+    <hyperlink ref="C45" r:id="rId43"/>
+    <hyperlink ref="C46" r:id="rId44"/>
+    <hyperlink ref="C47" r:id="rId45"/>
+    <hyperlink ref="C48" r:id="rId46"/>
+    <hyperlink ref="C49" r:id="rId47"/>
+    <hyperlink ref="C50" r:id="rId48"/>
+    <hyperlink ref="C51" r:id="rId49"/>
+    <hyperlink ref="C52" r:id="rId50"/>
+    <hyperlink ref="C53" r:id="rId51"/>
+    <hyperlink ref="C54" r:id="rId52"/>
+    <hyperlink ref="C55" r:id="rId53"/>
+    <hyperlink ref="C56" r:id="rId54"/>
+    <hyperlink ref="C57" r:id="rId55"/>
+    <hyperlink ref="C58" r:id="rId56"/>
+    <hyperlink ref="C59" r:id="rId57"/>
+    <hyperlink ref="C60" r:id="rId58"/>
+    <hyperlink ref="C62" r:id="rId59"/>
+    <hyperlink ref="C63" r:id="rId60"/>
+    <hyperlink ref="C64" r:id="rId61"/>
+    <hyperlink ref="C65" r:id="rId62"/>
+    <hyperlink ref="C66" r:id="rId63"/>
+    <hyperlink ref="C67" r:id="rId64"/>
+    <hyperlink ref="C68" r:id="rId65"/>
+    <hyperlink ref="C69" r:id="rId66"/>
+    <hyperlink ref="C70" r:id="rId67"/>
+    <hyperlink ref="C71" r:id="rId68"/>
+    <hyperlink ref="C72" r:id="rId69"/>
+    <hyperlink ref="C73" r:id="rId70"/>
+    <hyperlink ref="C74" r:id="rId71"/>
+    <hyperlink ref="C75" r:id="rId72"/>
+    <hyperlink ref="C76" r:id="rId73"/>
+    <hyperlink ref="C77" r:id="rId74"/>
+    <hyperlink ref="C78" r:id="rId75"/>
+    <hyperlink ref="C79" r:id="rId76"/>
+    <hyperlink ref="C80" r:id="rId77"/>
+    <hyperlink ref="C81" r:id="rId78"/>
+    <hyperlink ref="C82" r:id="rId79"/>
+    <hyperlink ref="C83" r:id="rId80"/>
+    <hyperlink ref="C84" r:id="rId81"/>
+    <hyperlink ref="C85" r:id="rId82"/>
+    <hyperlink ref="C86" r:id="rId83"/>
+    <hyperlink ref="C87" r:id="rId84"/>
+    <hyperlink ref="C88" r:id="rId85"/>
+    <hyperlink ref="C89" r:id="rId86"/>
+    <hyperlink ref="C90" r:id="rId87"/>
+    <hyperlink ref="C91" r:id="rId88"/>
+    <hyperlink ref="C92" r:id="rId89"/>
+    <hyperlink ref="C93" r:id="rId90"/>
+    <hyperlink ref="C95" r:id="rId91"/>
+    <hyperlink ref="C96" r:id="rId92"/>
+    <hyperlink ref="C97" r:id="rId93"/>
+    <hyperlink ref="C99" r:id="rId94"/>
+    <hyperlink ref="C101" r:id="rId95"/>
+    <hyperlink ref="C102" r:id="rId96"/>
+    <hyperlink ref="C103" r:id="rId97"/>
+    <hyperlink ref="C104" r:id="rId98"/>
+    <hyperlink ref="C105" r:id="rId99"/>
+    <hyperlink ref="C106" r:id="rId100"/>
   </hyperlinks>
-  <printOptions headings="0" gridLines="0" horizontalCentered="0" verticalCentered="0"/>
-  <pageMargins left="0.78750000000000009" right="0.78750000000000009" top="1.05277777777778" bottom="1.05277777777778" header="0.78750000000000009" footer="0.78750000000000009"/>
-  <pageSetup paperSize="1" scale="100" firstPageNumber="1" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="1" errors="displayed" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageMargins left="0.7875000000000001" right="0.7875000000000001" top="1.05277777777778" bottom="1.05277777777778" header="0.7875000000000001" footer="0.7875000000000001"/>
+  <pageSetup paperSize="1" orientation="portrait" horizontalDpi="300" verticalDpi="300" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" usePrinterDefaults="1" copies="1"/>
   <headerFooter>
     <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;A</oddHeader>
     <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12Page &amp;P</oddFooter>

</xml_diff>

<commit_message>
Minutes for 2026-06-05 (#181)
</commit_message>
<xml_diff>
--- a/data/wg_attendees.xlsx
+++ b/data/wg_attendees.xlsx
@@ -1,23 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <workbookPr date1904="0"/>
-  <workbookProtection/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
+  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <bookViews>
     <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet sheetId="1" name="Sheet1" state="visible" r:id="rId4"/>
   </sheets>
-  <calcPr refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.001"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{D0CA8CA8-9F24-4464-BF8E-62219DCF47F9}"/>
-  </extLst>
+  <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="196" uniqueCount="196">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="324" uniqueCount="202">
   <si>
     <t>name</t>
   </si>
@@ -28,13 +25,13 @@
     <t>affiliation_url</t>
   </si>
   <si>
-    <t xml:space="preserve">Joseph Rickert</t>
+    <t>Joseph Rickert</t>
   </si>
   <si>
     <t>Unknown</t>
   </si>
   <si>
-    <t xml:space="preserve">Adrian Waddell</t>
+    <t>Adrian Waddell</t>
   </si>
   <si>
     <t>Roche/Genentech</t>
@@ -43,13 +40,13 @@
     <t>https://www.gene.com</t>
   </si>
   <si>
-    <t xml:space="preserve">Doug Kelkhoff</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tadeusz Lewandowski</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ning Leng</t>
+    <t>Doug Kelkhoff</t>
+  </si>
+  <si>
+    <t>Tadeusz Lewandowski</t>
+  </si>
+  <si>
+    <t>Ning Leng</t>
   </si>
   <si>
     <t>AbbVie</t>
@@ -58,13 +55,13 @@
     <t>https://www.abbvie.com/</t>
   </si>
   <si>
-    <t xml:space="preserve">Heng Wang</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Beverly Chin</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bob Engle</t>
+    <t>Heng Wang</t>
+  </si>
+  <si>
+    <t>Beverly Chin</t>
+  </si>
+  <si>
+    <t>Bob Engle</t>
   </si>
   <si>
     <t>Biogen</t>
@@ -73,25 +70,25 @@
     <t xml:space="preserve">https://www.biogen.com/en_us/home.html </t>
   </si>
   <si>
-    <t xml:space="preserve">Christopher Kania</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Nate Mockler</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tim Powell</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Juliane Manitz</t>
-  </si>
-  <si>
-    <t xml:space="preserve">EMD Serono</t>
+    <t>Christopher Kania</t>
+  </si>
+  <si>
+    <t>Nate Mockler</t>
+  </si>
+  <si>
+    <t>Tim Powell</t>
+  </si>
+  <si>
+    <t>Juliane Manitz</t>
+  </si>
+  <si>
+    <t>EMD Serono</t>
   </si>
   <si>
     <t xml:space="preserve">https://www.emdserono.com/us-en </t>
   </si>
   <si>
-    <t xml:space="preserve">Lyn Taylor</t>
+    <t>Lyn Taylor</t>
   </si>
   <si>
     <t>Phastar</t>
@@ -100,7 +97,7 @@
     <t>https://phastar.com/</t>
   </si>
   <si>
-    <t xml:space="preserve">Mike Stackhouse</t>
+    <t>Mike Stackhouse</t>
   </si>
   <si>
     <t>Atorus</t>
@@ -109,10 +106,10 @@
     <t xml:space="preserve">https://www.atorusresearch.com/ </t>
   </si>
   <si>
-    <t xml:space="preserve">Eli Miller</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Paul Schuette</t>
+    <t>Eli Miller</t>
+  </si>
+  <si>
+    <t>Paul Schuette</t>
   </si>
   <si>
     <t>FDA</t>
@@ -121,28 +118,28 @@
     <t>https://www.fda.gov/</t>
   </si>
   <si>
-    <t xml:space="preserve">Ethan Chen</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bryant Chen</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Jiang Xu</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Jizu Zhi</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Kevin Snyder</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hye Soo Cho</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Maria Matilde Kam</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sascha Ahrweiler</t>
+    <t>Ethan Chen</t>
+  </si>
+  <si>
+    <t>Bryant Chen</t>
+  </si>
+  <si>
+    <t>Jiang Xu</t>
+  </si>
+  <si>
+    <t>Jizu Zhi</t>
+  </si>
+  <si>
+    <t>Kevin Snyder</t>
+  </si>
+  <si>
+    <t>Hye Soo Cho</t>
+  </si>
+  <si>
+    <t>Maria Matilde Kam</t>
+  </si>
+  <si>
+    <t>Sascha Ahrweiler</t>
   </si>
   <si>
     <t>Bayer</t>
@@ -151,7 +148,7 @@
     <t>https://www.bayer.com/en/</t>
   </si>
   <si>
-    <t xml:space="preserve">Phil Bowsher</t>
+    <t>Phil Bowsher</t>
   </si>
   <si>
     <t>Posit</t>
@@ -160,7 +157,7 @@
     <t xml:space="preserve">https://posit.co </t>
   </si>
   <si>
-    <t xml:space="preserve">Yilong Zhang</t>
+    <t>Yilong Zhang</t>
   </si>
   <si>
     <t>Meta</t>
@@ -169,7 +166,7 @@
     <t xml:space="preserve">https://facebook.com </t>
   </si>
   <si>
-    <t xml:space="preserve">Keaven Anderson</t>
+    <t>Keaven Anderson</t>
   </si>
   <si>
     <t>Merck</t>
@@ -178,10 +175,10 @@
     <t xml:space="preserve">https://www.merck.com </t>
   </si>
   <si>
-    <t xml:space="preserve">Nan Xiao</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Gregory Chen</t>
+    <t>Nan Xiao</t>
+  </si>
+  <si>
+    <t>Gregory Chen</t>
   </si>
   <si>
     <t>MSD</t>
@@ -190,13 +187,13 @@
     <t xml:space="preserve">https://www.msd.com/ </t>
   </si>
   <si>
-    <t xml:space="preserve">Miriam Fossati</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Peikun Wu</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Paulo Bargo</t>
+    <t>Miriam Fossati</t>
+  </si>
+  <si>
+    <t>Peikun Wu</t>
+  </si>
+  <si>
+    <t>Paulo Bargo</t>
   </si>
   <si>
     <t>Janssen</t>
@@ -205,7 +202,7 @@
     <t>https://www.jnjmedtech.com</t>
   </si>
   <si>
-    <t xml:space="preserve">Andy Nicholls</t>
+    <t>Andy Nicholls</t>
   </si>
   <si>
     <t>GSK</t>
@@ -214,16 +211,16 @@
     <t xml:space="preserve">https://www.gsk.com/en-gb/home/ </t>
   </si>
   <si>
-    <t xml:space="preserve">Ojesh Upandhyay</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ellis Hughes</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ben Straub</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Kevin Bolger</t>
+    <t>Ojesh Upandhyay</t>
+  </si>
+  <si>
+    <t>Ellis Hughes</t>
+  </si>
+  <si>
+    <t>Ben Straub</t>
+  </si>
+  <si>
+    <t>Kevin Bolger</t>
   </si>
   <si>
     <t>Procogia</t>
@@ -232,16 +229,16 @@
     <t xml:space="preserve">https://procogia.com </t>
   </si>
   <si>
-    <t xml:space="preserve">Eric Nantz</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Eli Lilly</t>
+    <t>Eric Nantz</t>
+  </si>
+  <si>
+    <t>Eli Lilly</t>
   </si>
   <si>
     <t xml:space="preserve">https://lilly.com </t>
   </si>
   <si>
-    <t xml:space="preserve">Bella Feng</t>
+    <t>Bella Feng</t>
   </si>
   <si>
     <t>EQRx</t>
@@ -250,22 +247,22 @@
     <t xml:space="preserve">https://www.eqrx.com </t>
   </si>
   <si>
-    <t xml:space="preserve">Steven Hasendinckx</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Johnson &amp; Johnson</t>
+    <t>Steven Hasendinckx</t>
+  </si>
+  <si>
+    <t>Johnson &amp; Johnson</t>
   </si>
   <si>
     <t>https://www.jnj.com</t>
   </si>
   <si>
-    <t xml:space="preserve">Heidi Curinckx</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Renping Zhang</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hong Yan</t>
+    <t>Heidi Curinckx</t>
+  </si>
+  <si>
+    <t>Renping Zhang</t>
+  </si>
+  <si>
+    <t>Hong Yan</t>
   </si>
   <si>
     <t>Regeneron</t>
@@ -274,16 +271,16 @@
     <t xml:space="preserve">https://www.regeneron.com </t>
   </si>
   <si>
-    <t xml:space="preserve">Ari Siggaard Knoph</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Novo Nordisk</t>
+    <t>Ari Siggaard Knoph</t>
+  </si>
+  <si>
+    <t>Novo Nordisk</t>
   </si>
   <si>
     <t xml:space="preserve">https://www.novonordisk.com/ </t>
   </si>
   <si>
-    <t xml:space="preserve">Michael Blanks</t>
+    <t>Michael Blanks</t>
   </si>
   <si>
     <t>BeiGene</t>
@@ -292,28 +289,28 @@
     <t xml:space="preserve">https://www.beigene.com/ </t>
   </si>
   <si>
-    <t xml:space="preserve">Robert Devine</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ryan Johnson</t>
+    <t>Robert Devine</t>
+  </si>
+  <si>
+    <t>Ryan Johnson</t>
   </si>
   <si>
     <t xml:space="preserve">https://posit.co  </t>
   </si>
   <si>
-    <t xml:space="preserve">Emily Nguyan</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Frederic Saad</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Jonathan Tisack</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hao Wang</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Graeme Hickey</t>
+    <t>Emily Nguyan</t>
+  </si>
+  <si>
+    <t>Frederic Saad</t>
+  </si>
+  <si>
+    <t>Jonathan Tisack</t>
+  </si>
+  <si>
+    <t>Hao Wang</t>
+  </si>
+  <si>
+    <t>Graeme Hickey</t>
   </si>
   <si>
     <t>Metronic</t>
@@ -322,19 +319,19 @@
     <t xml:space="preserve">https://www.medtronic.com/us-en/index.html </t>
   </si>
   <si>
-    <t xml:space="preserve">Michael Mayer</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Xin Qiu</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Shannon Lewis</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Joel Laxamana</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Stephanie Lussier</t>
+    <t>Michael Mayer</t>
+  </si>
+  <si>
+    <t>Xin Qiu</t>
+  </si>
+  <si>
+    <t>Shannon Lewis</t>
+  </si>
+  <si>
+    <t>Joel Laxamana</t>
+  </si>
+  <si>
+    <t>Stephanie Lussier</t>
   </si>
   <si>
     <t>Moderna</t>
@@ -343,10 +340,10 @@
     <t xml:space="preserve">https://www.modernatx.com </t>
   </si>
   <si>
-    <t xml:space="preserve">Thomas Neitmann</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sam Parmar</t>
+    <t>Thomas Neitmann</t>
+  </si>
+  <si>
+    <t>Sam Parmar</t>
   </si>
   <si>
     <t>Pfizer</t>
@@ -355,10 +352,10 @@
     <t xml:space="preserve">https://www.pfizer.com/ </t>
   </si>
   <si>
-    <t xml:space="preserve">Brian Sucher</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dadong Zhang</t>
+    <t>Brian Sucher</t>
+  </si>
+  <si>
+    <t>Dadong Zhang</t>
   </si>
   <si>
     <t>Illumina</t>
@@ -367,16 +364,16 @@
     <t xml:space="preserve">https://www.illumina.com/ </t>
   </si>
   <si>
-    <t xml:space="preserve">Yutong Liu</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lei Zhao</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Honghong Zhou</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Saghir Bashir</t>
+    <t>Yutong Liu</t>
+  </si>
+  <si>
+    <t>Lei Zhao</t>
+  </si>
+  <si>
+    <t>Honghong Zhou</t>
+  </si>
+  <si>
+    <t>Saghir Bashir</t>
   </si>
   <si>
     <t>Argenx</t>
@@ -385,109 +382,109 @@
     <t xml:space="preserve">https://www.argenx.com/ </t>
   </si>
   <si>
-    <t xml:space="preserve">Sean Healey</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Gabriel Becker</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Rupam Bhattacharyya</t>
-  </si>
-  <si>
-    <t xml:space="preserve">University of Michigan</t>
+    <t>Sean Healey</t>
+  </si>
+  <si>
+    <t>Gabriel Becker</t>
+  </si>
+  <si>
+    <t>Rupam Bhattacharyya</t>
+  </si>
+  <si>
+    <t>University of Michigan</t>
   </si>
   <si>
     <t xml:space="preserve">https://publichealth.umich.edu/ </t>
   </si>
   <si>
-    <t xml:space="preserve">Helena Sviglin</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Neetu Sangari</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Phanikumar Tata</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Syneos Health</t>
+    <t>Helena Sviglin</t>
+  </si>
+  <si>
+    <t>Neetu Sangari</t>
+  </si>
+  <si>
+    <t>Phanikumar Tata</t>
+  </si>
+  <si>
+    <t>Syneos Health</t>
   </si>
   <si>
     <t xml:space="preserve">https://www.syneoshealth.com/ </t>
   </si>
   <si>
-    <t xml:space="preserve">Kui Schen</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Estella Dong</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Yiwen Luo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bryan Tegomoh</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CDC Foundation</t>
+    <t>Kui Schen</t>
+  </si>
+  <si>
+    <t>Estella Dong</t>
+  </si>
+  <si>
+    <t>Yiwen Luo</t>
+  </si>
+  <si>
+    <t>Bryan Tegomoh</t>
+  </si>
+  <si>
+    <t>CDC Foundation</t>
   </si>
   <si>
     <t xml:space="preserve">https://www.cdcfoundation.org/ </t>
   </si>
   <si>
-    <t xml:space="preserve">Coline Zeballos</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Luke Schantz</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R Consortium</t>
+    <t>Coline Zeballos</t>
+  </si>
+  <si>
+    <t>Luke Schantz</t>
+  </si>
+  <si>
+    <t>R Consortium</t>
   </si>
   <si>
     <t>https://www.r-consortium.org</t>
   </si>
   <si>
-    <t xml:space="preserve">Andrew Borgman</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bristol Myers Squibb</t>
+    <t>Andrew Borgman</t>
+  </si>
+  <si>
+    <t>Bristol Myers Squibb</t>
   </si>
   <si>
     <t xml:space="preserve">https://www.bms.com/ </t>
   </si>
   <si>
-    <t xml:space="preserve">Henry Wang</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Chenguang Wang</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Qin Lin</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Kevin Kunzmann</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Boehringer Ingelheim</t>
+    <t>Henry Wang</t>
+  </si>
+  <si>
+    <t>Chenguang Wang</t>
+  </si>
+  <si>
+    <t>Qin Lin</t>
+  </si>
+  <si>
+    <t>Kevin Kunzmann</t>
+  </si>
+  <si>
+    <t>Boehringer Ingelheim</t>
   </si>
   <si>
     <t xml:space="preserve">https://www.boehringer-ingelheim.com/ </t>
   </si>
   <si>
-    <t xml:space="preserve">Michael Kane</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MD Anderson Cancer Institute</t>
+    <t>Michael Kane</t>
+  </si>
+  <si>
+    <t>MD Anderson Cancer Institute</t>
   </si>
   <si>
     <t xml:space="preserve">https://www.mdanderson.org/ </t>
   </si>
   <si>
-    <t xml:space="preserve">Terry Christiani</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Amanda Martin</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Andre Couturier</t>
+    <t>Terry Christiani</t>
+  </si>
+  <si>
+    <t>Amanda Martin</t>
+  </si>
+  <si>
+    <t>Andre Couturier</t>
   </si>
   <si>
     <t>Sanofi</t>
@@ -496,13 +493,13 @@
     <t xml:space="preserve">https://www.sanofi.com/ </t>
   </si>
   <si>
-    <t xml:space="preserve">Nicholas Masel</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lovemore Gakava</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Katie Harding</t>
+    <t>Nicholas Masel</t>
+  </si>
+  <si>
+    <t>Lovemore Gakava</t>
+  </si>
+  <si>
+    <t>Katie Harding</t>
   </si>
   <si>
     <t>Freenome</t>
@@ -511,10 +508,10 @@
     <t xml:space="preserve">https://www.freenome.com/ </t>
   </si>
   <si>
-    <t xml:space="preserve">Youn Kyeong Chang</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sam Hume</t>
+    <t>Youn Kyeong Chang</t>
+  </si>
+  <si>
+    <t>Sam Hume</t>
   </si>
   <si>
     <t>CDISC</t>
@@ -523,7 +520,7 @@
     <t xml:space="preserve">https://www.cdisc.org/ </t>
   </si>
   <si>
-    <t xml:space="preserve">Camille Calmasini</t>
+    <t>Camille Calmasini</t>
   </si>
   <si>
     <t>Natera</t>
@@ -532,52 +529,55 @@
     <t>https://www.natera.com/</t>
   </si>
   <si>
-    <t xml:space="preserve">Jim Rothstein</t>
+    <t>Jim Rothstein</t>
   </si>
   <si>
     <t>Freelance</t>
   </si>
   <si>
-    <t xml:space="preserve">Nabil Baugher</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Baseline AI</t>
+    <t>Nabil Baugher</t>
+  </si>
+  <si>
+    <t>Baseline AI</t>
   </si>
   <si>
     <t>https://www.baselinetrials.com</t>
   </si>
   <si>
-    <t xml:space="preserve">Gabriel Krotkov</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hong Zheng</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Karthik Velega</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Luis Osorio</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Los Angeles Count Department of Public Health</t>
+    <t>Gabriel Krotkov</t>
+  </si>
+  <si>
+    <t>Hong Zheng</t>
+  </si>
+  <si>
+    <t>Karthik Velega</t>
+  </si>
+  <si>
+    <t>Luis Osorio</t>
+  </si>
+  <si>
+    <t>Los Angeles Count Department of Public Health</t>
   </si>
   <si>
     <t>http://publichealth.lacounty.gov/</t>
   </si>
   <si>
-    <t xml:space="preserve">Sara Z</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sydney Dennison</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Vital Reddy Jaggavarapu</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Yogesh Gupta</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Jared Woolfolk</t>
+    <t>Sarah Zanzoul</t>
+  </si>
+  <si>
+    <t>https://www.pfizer.com/</t>
+  </si>
+  <si>
+    <t>Sydney Dennison</t>
+  </si>
+  <si>
+    <t>Vital Reddy Jaggavarapu</t>
+  </si>
+  <si>
+    <t>Yogesh Gupta</t>
+  </si>
+  <si>
+    <t>Jared Woolfolk</t>
   </si>
   <si>
     <t>Cytel</t>
@@ -586,50 +586,68 @@
     <t>https://cytel.com/</t>
   </si>
   <si>
-    <t xml:space="preserve">Vinod Kumar</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TruMines Clinical</t>
+    <t>Vinod Kumar</t>
+  </si>
+  <si>
+    <t>TruMines Clinical</t>
   </si>
   <si>
     <t>https://trumindsclinical.com/</t>
   </si>
   <si>
-    <t xml:space="preserve">Chi-Hua Huang</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Astellas Pharmaceuticals</t>
+    <t>Chi-Hua Huang</t>
+  </si>
+  <si>
+    <t>Astellas Pharmaceuticals</t>
   </si>
   <si>
     <t>https://www.astellas.com/en/</t>
   </si>
   <si>
     <t>Ram</t>
+  </si>
+  <si>
+    <t>Brandon Sucher</t>
+  </si>
+  <si>
+    <t>https://www.modernatx.com/</t>
+  </si>
+  <si>
+    <t>Dmitry Kolosov</t>
+  </si>
+  <si>
+    <t>Vital Jaggavarapu</t>
+  </si>
+  <si>
+    <t>https://www.boehringer-ingelheim.com/</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="4">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
-      <sz val="10.000000"/>
       <color theme="1"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <color theme="1"/>
+      <sz val="10"/>
       <name val="Arial"/>
     </font>
     <font>
-      <sz val="10.000000"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10.000000"/>
       <color indexed="4"/>
+      <sz val="10"/>
       <name val="Arial"/>
     </font>
     <font>
       <u/>
-      <sz val="10.000000"/>
       <color theme="10"/>
+      <sz val="10"/>
       <name val="Arial"/>
     </font>
   </fonts>
@@ -641,7 +659,14 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
     <border>
       <left style="none"/>
       <right style="none"/>
@@ -650,46 +675,26 @@
       <diagonal style="none"/>
     </border>
   </borders>
-  <cellStyleXfs count="6">
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
-      <protection hidden="0" locked="1"/>
-    </xf>
-    <xf fontId="1" fillId="0" borderId="0" numFmtId="43" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyProtection="0"/>
-    <xf fontId="1" fillId="0" borderId="0" numFmtId="41" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyProtection="0"/>
-    <xf fontId="1" fillId="0" borderId="0" numFmtId="44" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyProtection="0"/>
-    <xf fontId="1" fillId="0" borderId="0" numFmtId="42" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyProtection="0"/>
-    <xf fontId="1" fillId="0" borderId="0" numFmtId="9" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyProtection="0"/>
+  <cellStyleXfs count="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyProtection="0">
-      <protection hidden="0" locked="1"/>
-    </xf>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyProtection="1">
-      <protection hidden="0" locked="1"/>
-    </xf>
-    <xf fontId="2" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyProtection="1">
-      <protection hidden="0" locked="1"/>
-    </xf>
-    <xf fontId="3" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyProtection="1">
-      <protection hidden="0" locked="1"/>
-    </xf>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyProtection="1">
-      <protection hidden="0" locked="1"/>
-    </xf>
+  <cellXfs count="4">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
-  <cellStyles count="6">
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Comma" xfId="1" builtinId="3"/>
-    <cellStyle name="Comma [0]" xfId="2" builtinId="6"/>
-    <cellStyle name="Currency" xfId="3" builtinId="4"/>
-    <cellStyle name="Currency [0]" xfId="4" builtinId="7"/>
-    <cellStyle name="Percent" xfId="5" builtinId="5"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
@@ -1104,19 +1109,19 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
-  <sheetPr filterMode="0">
-    <outlinePr applyStyles="0" summaryBelow="1" summaryRight="1" showOutlineSymbols="1"/>
-    <pageSetUpPr autoPageBreaks="1" fitToPage="0"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <sheetFormatPr defaultColWidth="11.60546875" defaultRowHeight="15"/>
+  <dimension ref="A1:C110"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="11.60546875"/>
   <cols>
-    <col customWidth="1" min="1" max="1" style="1" width="28.109999999999999"/>
-    <col customWidth="1" min="2" max="2" style="1" width="38.50390625"/>
-    <col customWidth="1" min="3" max="3" style="1" width="36.299999999999997"/>
+    <col min="1" max="1" width="28.11" style="1" customWidth="1"/>
+    <col min="2" max="2" width="38.50390625" style="1" customWidth="1"/>
+    <col min="3" max="3" width="36.3" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="12.800000000000001">
+    <row r="1" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1127,7 +1132,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" ht="12.800000000000001">
+    <row r="2" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>3</v>
       </c>
@@ -1136,7 +1141,7 @@
       </c>
       <c r="C2" s="2"/>
     </row>
-    <row r="3" ht="12.800000000000001">
+    <row r="3" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>5</v>
       </c>
@@ -1147,7 +1152,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="4" ht="12.800000000000001">
+    <row r="4" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>8</v>
       </c>
@@ -1158,7 +1163,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="5" ht="12.800000000000001">
+    <row r="5" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>9</v>
       </c>
@@ -1169,7 +1174,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="6" ht="12.800000000000001">
+    <row r="6" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>10</v>
       </c>
@@ -1180,7 +1185,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="7" ht="12.800000000000001">
+    <row r="7" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>13</v>
       </c>
@@ -1191,7 +1196,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="8" ht="12.800000000000001">
+    <row r="8" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>14</v>
       </c>
@@ -1202,7 +1207,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="9" ht="12.800000000000001">
+    <row r="9" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>15</v>
       </c>
@@ -1213,7 +1218,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="10" ht="12.800000000000001">
+    <row r="10" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>18</v>
       </c>
@@ -1224,7 +1229,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="11" ht="12.800000000000001">
+    <row r="11" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>19</v>
       </c>
@@ -1235,7 +1240,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="12" ht="12.800000000000001">
+    <row r="12" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>20</v>
       </c>
@@ -1246,7 +1251,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="13" ht="12.800000000000001">
+    <row r="13" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
         <v>21</v>
       </c>
@@ -1257,7 +1262,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="14" ht="12.800000000000001">
+    <row r="14" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
         <v>24</v>
       </c>
@@ -1268,7 +1273,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="15" ht="12.800000000000001">
+    <row r="15" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
         <v>27</v>
       </c>
@@ -1279,7 +1284,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="16" ht="12.800000000000001">
+    <row r="16" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
         <v>30</v>
       </c>
@@ -1290,7 +1295,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="17" ht="12.800000000000001">
+    <row r="17" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
         <v>31</v>
       </c>
@@ -1301,7 +1306,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="18" ht="12.800000000000001">
+    <row r="18" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
         <v>34</v>
       </c>
@@ -1312,7 +1317,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="19" ht="12.800000000000001">
+    <row r="19" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
         <v>35</v>
       </c>
@@ -1323,7 +1328,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="20" ht="12.800000000000001">
+    <row r="20" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
         <v>36</v>
       </c>
@@ -1334,7 +1339,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="21" ht="12.800000000000001">
+    <row r="21" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
         <v>37</v>
       </c>
@@ -1345,7 +1350,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="22" ht="12.800000000000001">
+    <row r="22" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
         <v>38</v>
       </c>
@@ -1356,7 +1361,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="23" ht="12.800000000000001">
+    <row r="23" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
         <v>39</v>
       </c>
@@ -1367,7 +1372,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="24" ht="12.800000000000001">
+    <row r="24" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
         <v>40</v>
       </c>
@@ -1378,7 +1383,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="25" ht="12.800000000000001">
+    <row r="25" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
         <v>41</v>
       </c>
@@ -1389,7 +1394,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="26" ht="12.800000000000001">
+    <row r="26" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
         <v>44</v>
       </c>
@@ -1400,7 +1405,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="27" ht="12.800000000000001">
+    <row r="27" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
         <v>47</v>
       </c>
@@ -1411,7 +1416,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="28" ht="12.800000000000001">
+    <row r="28" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
         <v>50</v>
       </c>
@@ -1422,7 +1427,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="29" ht="12.800000000000001">
+    <row r="29" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" s="1" t="s">
         <v>53</v>
       </c>
@@ -1433,7 +1438,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="30" ht="12.800000000000001">
+    <row r="30" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30" s="1" t="s">
         <v>54</v>
       </c>
@@ -1444,7 +1449,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="31" ht="12.800000000000001">
+    <row r="31" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A31" s="1" t="s">
         <v>57</v>
       </c>
@@ -1455,7 +1460,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="32" ht="12.800000000000001">
+    <row r="32" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A32" s="1" t="s">
         <v>58</v>
       </c>
@@ -1466,7 +1471,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="33" ht="12.800000000000001">
+    <row r="33" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A33" s="1" t="s">
         <v>59</v>
       </c>
@@ -1477,7 +1482,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="34" ht="12.800000000000001">
+    <row r="34" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A34" s="1" t="s">
         <v>62</v>
       </c>
@@ -1488,7 +1493,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="35" ht="12.800000000000001">
+    <row r="35" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A35" s="1" t="s">
         <v>65</v>
       </c>
@@ -1499,7 +1504,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="36" ht="12.800000000000001">
+    <row r="36" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A36" s="1" t="s">
         <v>66</v>
       </c>
@@ -1510,7 +1515,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="37" ht="12.800000000000001">
+    <row r="37" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A37" s="1" t="s">
         <v>67</v>
       </c>
@@ -1521,7 +1526,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="38" ht="12.800000000000001">
+    <row r="38" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A38" s="1" t="s">
         <v>68</v>
       </c>
@@ -1532,7 +1537,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="39" ht="12.800000000000001">
+    <row r="39" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A39" s="1" t="s">
         <v>71</v>
       </c>
@@ -1543,7 +1548,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="40" ht="12.800000000000001">
+    <row r="40" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A40" s="1" t="s">
         <v>74</v>
       </c>
@@ -1554,7 +1559,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="41" ht="12.800000000000001">
+    <row r="41" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A41" s="1" t="s">
         <v>77</v>
       </c>
@@ -1565,7 +1570,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="42" ht="12.800000000000001">
+    <row r="42" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A42" s="1" t="s">
         <v>80</v>
       </c>
@@ -1576,7 +1581,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="43" ht="12.800000000000001">
+    <row r="43" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A43" s="1" t="s">
         <v>81</v>
       </c>
@@ -1587,7 +1592,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="44" ht="12.800000000000001">
+    <row r="44" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A44" s="1" t="s">
         <v>82</v>
       </c>
@@ -1598,7 +1603,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="45" ht="12.800000000000001">
+    <row r="45" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A45" s="1" t="s">
         <v>85</v>
       </c>
@@ -1609,7 +1614,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="46" ht="12.800000000000001">
+    <row r="46" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A46" s="1" t="s">
         <v>88</v>
       </c>
@@ -1620,7 +1625,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="47" ht="12.800000000000001">
+    <row r="47" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A47" s="1" t="s">
         <v>91</v>
       </c>
@@ -1631,7 +1636,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="48" ht="12.800000000000001">
+    <row r="48" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A48" s="1" t="s">
         <v>92</v>
       </c>
@@ -1642,7 +1647,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="49" ht="12.800000000000001">
+    <row r="49" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A49" s="1" t="s">
         <v>94</v>
       </c>
@@ -1653,7 +1658,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="50" ht="12.800000000000001">
+    <row r="50" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A50" s="1" t="s">
         <v>95</v>
       </c>
@@ -1664,7 +1669,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="51" ht="12.800000000000001">
+    <row r="51" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A51" s="1" t="s">
         <v>96</v>
       </c>
@@ -1675,7 +1680,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="52" ht="12.800000000000001">
+    <row r="52" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A52" s="1" t="s">
         <v>97</v>
       </c>
@@ -1686,7 +1691,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="53" ht="12.800000000000001">
+    <row r="53" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A53" s="1" t="s">
         <v>98</v>
       </c>
@@ -1697,7 +1702,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="54" ht="12.800000000000001">
+    <row r="54" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A54" s="1" t="s">
         <v>101</v>
       </c>
@@ -1708,7 +1713,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="55" ht="12.800000000000001">
+    <row r="55" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A55" s="1" t="s">
         <v>102</v>
       </c>
@@ -1719,7 +1724,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="56" ht="12.800000000000001">
+    <row r="56" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A56" s="1" t="s">
         <v>103</v>
       </c>
@@ -1730,7 +1735,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="57" ht="12.800000000000001">
+    <row r="57" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A57" s="1" t="s">
         <v>104</v>
       </c>
@@ -1741,7 +1746,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="58" ht="12.800000000000001">
+    <row r="58" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A58" s="1" t="s">
         <v>105</v>
       </c>
@@ -1752,7 +1757,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="59" ht="12.800000000000001">
+    <row r="59" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A59" s="1" t="s">
         <v>108</v>
       </c>
@@ -1763,7 +1768,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="60" ht="12.800000000000001">
+    <row r="60" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A60" s="1" t="s">
         <v>109</v>
       </c>
@@ -1774,7 +1779,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="61" ht="12.800000000000001">
+    <row r="61" ht="12.8" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A61" s="1" t="s">
         <v>112</v>
       </c>
@@ -1782,7 +1787,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="62" ht="12.800000000000001">
+    <row r="62" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A62" s="1" t="s">
         <v>113</v>
       </c>
@@ -1793,7 +1798,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="63" ht="12.800000000000001">
+    <row r="63" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A63" s="1" t="s">
         <v>116</v>
       </c>
@@ -1804,7 +1809,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="64" ht="12.800000000000001">
+    <row r="64" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A64" s="1" t="s">
         <v>117</v>
       </c>
@@ -1815,7 +1820,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="65" ht="12.800000000000001">
+    <row r="65" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A65" s="1" t="s">
         <v>118</v>
       </c>
@@ -1826,7 +1831,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="66" ht="12.800000000000001">
+    <row r="66" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A66" s="1" t="s">
         <v>119</v>
       </c>
@@ -1837,7 +1842,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="67" ht="12.800000000000001">
+    <row r="67" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A67" s="1" t="s">
         <v>122</v>
       </c>
@@ -1848,7 +1853,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="68" ht="12.800000000000001">
+    <row r="68" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A68" s="1" t="s">
         <v>123</v>
       </c>
@@ -1859,7 +1864,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="69" ht="12.800000000000001">
+    <row r="69" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A69" s="1" t="s">
         <v>124</v>
       </c>
@@ -1870,7 +1875,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="70" ht="12.800000000000001">
+    <row r="70" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A70" s="1" t="s">
         <v>127</v>
       </c>
@@ -1881,7 +1886,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="71" ht="12.800000000000001">
+    <row r="71" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A71" s="1" t="s">
         <v>128</v>
       </c>
@@ -1892,7 +1897,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="72" ht="12.800000000000001">
+    <row r="72" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A72" s="1" t="s">
         <v>129</v>
       </c>
@@ -1903,7 +1908,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="73" ht="12.800000000000001">
+    <row r="73" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A73" s="1" t="s">
         <v>132</v>
       </c>
@@ -1914,7 +1919,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="74" ht="12.800000000000001">
+    <row r="74" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A74" s="1" t="s">
         <v>133</v>
       </c>
@@ -1925,7 +1930,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="75" ht="12.800000000000001">
+    <row r="75" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A75" s="1" t="s">
         <v>134</v>
       </c>
@@ -1936,7 +1941,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="76" ht="12.800000000000001">
+    <row r="76" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A76" s="1" t="s">
         <v>135</v>
       </c>
@@ -1947,7 +1952,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="77" ht="12.800000000000001">
+    <row r="77" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A77" s="1" t="s">
         <v>138</v>
       </c>
@@ -1958,7 +1963,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="78" ht="12.800000000000001">
+    <row r="78" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A78" s="1" t="s">
         <v>139</v>
       </c>
@@ -1969,7 +1974,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="79" ht="12.800000000000001">
+    <row r="79" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A79" s="1" t="s">
         <v>142</v>
       </c>
@@ -1980,7 +1985,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="80" ht="12.800000000000001">
+    <row r="80" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A80" s="1" t="s">
         <v>145</v>
       </c>
@@ -1991,7 +1996,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="81" ht="12.800000000000001">
+    <row r="81" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A81" s="1" t="s">
         <v>146</v>
       </c>
@@ -2002,7 +2007,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="82" ht="12.800000000000001">
+    <row r="82" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A82" s="1" t="s">
         <v>147</v>
       </c>
@@ -2013,7 +2018,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="83" ht="12.800000000000001">
+    <row r="83" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A83" s="1" t="s">
         <v>148</v>
       </c>
@@ -2024,7 +2029,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="84" ht="12.800000000000001">
+    <row r="84" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A84" s="1" t="s">
         <v>151</v>
       </c>
@@ -2035,7 +2040,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="85" ht="12.800000000000001">
+    <row r="85" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A85" s="1" t="s">
         <v>154</v>
       </c>
@@ -2046,7 +2051,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="86" ht="12.800000000000001">
+    <row r="86" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A86" s="1" t="s">
         <v>155</v>
       </c>
@@ -2057,7 +2062,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="87" ht="12.800000000000001">
+    <row r="87" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A87" s="1" t="s">
         <v>156</v>
       </c>
@@ -2068,7 +2073,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="88" ht="12.800000000000001">
+    <row r="88" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A88" s="1" t="s">
         <v>159</v>
       </c>
@@ -2079,7 +2084,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="89" ht="12.800000000000001">
+    <row r="89" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A89" s="1" t="s">
         <v>160</v>
       </c>
@@ -2090,7 +2095,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="90" ht="12.800000000000001">
+    <row r="90" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A90" s="1" t="s">
         <v>161</v>
       </c>
@@ -2101,7 +2106,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="91" ht="12.800000000000001">
+    <row r="91" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A91" s="1" t="s">
         <v>164</v>
       </c>
@@ -2112,7 +2117,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="92" ht="12.800000000000001">
+    <row r="92" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A92" s="1" t="s">
         <v>165</v>
       </c>
@@ -2123,7 +2128,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="93" ht="12.800000000000001">
+    <row r="93" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A93" s="1" t="s">
         <v>168</v>
       </c>
@@ -2134,7 +2139,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="94" ht="12.800000000000001">
+    <row r="94" ht="12.8" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A94" s="1" t="s">
         <v>171</v>
       </c>
@@ -2142,7 +2147,7 @@
         <v>172</v>
       </c>
     </row>
-    <row r="95" ht="12.800000000000001">
+    <row r="95" ht="12.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A95" s="1" t="s">
         <v>173</v>
       </c>
@@ -2153,7 +2158,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="96" ht="15">
+    <row r="96" ht="15" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A96" s="1" t="s">
         <v>176</v>
       </c>
@@ -2164,7 +2169,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="97" ht="15">
+    <row r="97" ht="15" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A97" s="1" t="s">
         <v>177</v>
       </c>
@@ -2175,7 +2180,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="98" ht="15">
+    <row r="98" ht="15" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A98" s="1" t="s">
         <v>178</v>
       </c>
@@ -2183,7 +2188,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="99" ht="15">
+    <row r="99" ht="15" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A99" s="1" t="s">
         <v>179</v>
       </c>
@@ -2194,17 +2199,20 @@
         <v>181</v>
       </c>
     </row>
-    <row r="100" ht="15">
+    <row r="100" ht="15" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A100" s="1" t="s">
         <v>182</v>
       </c>
       <c r="B100" s="1" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="101" ht="15">
+        <v>110</v>
+      </c>
+      <c r="C100" s="1" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="101" ht="15" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A101" s="1" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="B101" s="1" t="s">
         <v>110</v>
@@ -2213,9 +2221,9 @@
         <v>111</v>
       </c>
     </row>
-    <row r="102" ht="15">
+    <row r="102" ht="15" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A102" s="1" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="B102" s="1" t="s">
         <v>149</v>
@@ -2224,9 +2232,9 @@
         <v>150</v>
       </c>
     </row>
-    <row r="103" ht="15">
+    <row r="103" ht="15" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A103" s="1" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="B103" s="1" t="s">
         <v>110</v>
@@ -2235,153 +2243,182 @@
         <v>111</v>
       </c>
     </row>
-    <row r="104" ht="15">
+    <row r="104" ht="15" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A104" s="1" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="B104" s="1" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="C104" s="3" t="s">
-        <v>188</v>
-      </c>
-    </row>
-    <row r="105" ht="15">
-      <c r="A105" s="4" t="s">
         <v>189</v>
       </c>
-      <c r="B105" s="4" t="s">
+    </row>
+    <row r="105" ht="15" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A105" s="1" t="s">
         <v>190</v>
       </c>
+      <c r="B105" s="1" t="s">
+        <v>191</v>
+      </c>
       <c r="C105" s="3" t="s">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="106" ht="15">
-      <c r="A106" s="4" t="s">
         <v>192</v>
       </c>
-      <c r="B106" s="4" t="s">
+    </row>
+    <row r="106" ht="15" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A106" s="1" t="s">
         <v>193</v>
       </c>
+      <c r="B106" s="1" t="s">
+        <v>194</v>
+      </c>
       <c r="C106" s="3" t="s">
-        <v>194</v>
-      </c>
-    </row>
-    <row r="107" ht="15">
-      <c r="A107" s="4" t="s">
         <v>195</v>
       </c>
-      <c r="B107" s="4" t="s">
+    </row>
+    <row r="107" ht="15" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A107" s="1" t="s">
+        <v>196</v>
+      </c>
+      <c r="B107" s="1" t="s">
         <v>4</v>
+      </c>
+    </row>
+    <row r="108" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A108" s="1" t="s">
+        <v>197</v>
+      </c>
+      <c r="B108" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="C108" s="1" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="109" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A109" s="1" t="s">
+        <v>199</v>
+      </c>
+      <c r="B109" s="1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="110" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A110" s="1" t="s">
+        <v>200</v>
+      </c>
+      <c r="B110" s="1" t="s">
+        <v>149</v>
+      </c>
+      <c r="C110" s="1" t="s">
+        <v>201</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink r:id="rId1" ref="C3"/>
-    <hyperlink r:id="rId1" ref="C4"/>
-    <hyperlink r:id="rId1" ref="C5"/>
-    <hyperlink r:id="rId2" ref="C6"/>
-    <hyperlink r:id="rId1" ref="C7"/>
-    <hyperlink r:id="rId1" ref="C8"/>
-    <hyperlink r:id="rId3" ref="C9"/>
-    <hyperlink r:id="rId3" ref="C10"/>
-    <hyperlink r:id="rId3" ref="C11"/>
-    <hyperlink r:id="rId3" ref="C12"/>
-    <hyperlink r:id="rId4" ref="C13"/>
-    <hyperlink r:id="rId5" ref="C14"/>
-    <hyperlink r:id="rId6" ref="C15"/>
-    <hyperlink r:id="rId6" ref="C16"/>
-    <hyperlink r:id="rId7" ref="C17"/>
-    <hyperlink r:id="rId7" ref="C18"/>
-    <hyperlink r:id="rId7" ref="C19"/>
-    <hyperlink r:id="rId7" ref="C20"/>
-    <hyperlink r:id="rId7" ref="C21"/>
-    <hyperlink r:id="rId7" ref="C22"/>
-    <hyperlink r:id="rId7" ref="C23"/>
-    <hyperlink r:id="rId7" ref="C24"/>
-    <hyperlink r:id="rId8" ref="C25"/>
-    <hyperlink r:id="rId9" ref="C26"/>
-    <hyperlink r:id="rId10" ref="C27"/>
-    <hyperlink r:id="rId11" ref="C28"/>
-    <hyperlink r:id="rId11" ref="C29"/>
-    <hyperlink r:id="rId12" ref="C30"/>
-    <hyperlink r:id="rId11" ref="C31"/>
-    <hyperlink r:id="rId11" ref="C32"/>
-    <hyperlink r:id="rId13" ref="C33"/>
-    <hyperlink r:id="rId14" ref="C34"/>
-    <hyperlink r:id="rId14" ref="C35"/>
-    <hyperlink r:id="rId14" ref="C36"/>
-    <hyperlink r:id="rId14" ref="C37"/>
-    <hyperlink r:id="rId15" ref="C38"/>
-    <hyperlink r:id="rId16" ref="C39"/>
-    <hyperlink r:id="rId17" ref="C40"/>
-    <hyperlink r:id="rId18" ref="C41"/>
-    <hyperlink r:id="rId18" ref="C42"/>
-    <hyperlink r:id="rId18" ref="C43"/>
-    <hyperlink r:id="rId19" ref="C44"/>
-    <hyperlink r:id="rId20" ref="C45"/>
-    <hyperlink r:id="rId21" ref="C46"/>
-    <hyperlink r:id="rId18" ref="C47"/>
-    <hyperlink r:id="rId9" ref="C48"/>
-    <hyperlink r:id="rId7" ref="C49"/>
-    <hyperlink r:id="rId13" ref="C50"/>
-    <hyperlink r:id="rId21" ref="C51"/>
-    <hyperlink r:id="rId7" ref="C52"/>
-    <hyperlink r:id="rId22" ref="C53"/>
-    <hyperlink r:id="rId9" ref="C54"/>
-    <hyperlink r:id="rId18" ref="C55"/>
-    <hyperlink r:id="rId21" ref="C56"/>
-    <hyperlink r:id="rId1" ref="C57"/>
-    <hyperlink r:id="rId23" ref="C58"/>
-    <hyperlink r:id="rId1" ref="C59"/>
-    <hyperlink r:id="rId24" ref="C60"/>
-    <hyperlink r:id="rId25" ref="C62"/>
-    <hyperlink r:id="rId23" ref="C63"/>
-    <hyperlink r:id="rId1" ref="C64"/>
-    <hyperlink r:id="rId23" ref="C65"/>
-    <hyperlink r:id="rId26" ref="C66"/>
-    <hyperlink r:id="rId24" ref="C67"/>
-    <hyperlink r:id="rId1" ref="C68"/>
-    <hyperlink r:id="rId27" ref="C69"/>
-    <hyperlink r:id="rId7" ref="C70"/>
-    <hyperlink r:id="rId24" ref="C71"/>
-    <hyperlink r:id="rId28" ref="C72"/>
-    <hyperlink r:id="rId8" ref="C73"/>
-    <hyperlink r:id="rId8" ref="C74"/>
-    <hyperlink r:id="rId11" ref="C75"/>
-    <hyperlink r:id="rId29" ref="C76"/>
-    <hyperlink r:id="rId1" ref="C77"/>
-    <hyperlink r:id="rId30" ref="C78"/>
-    <hyperlink r:id="rId31" ref="C79"/>
-    <hyperlink r:id="rId1" ref="C80"/>
-    <hyperlink r:id="rId19" ref="C81"/>
-    <hyperlink r:id="rId14" ref="C82"/>
-    <hyperlink r:id="rId32" ref="C83"/>
-    <hyperlink r:id="rId33" ref="C84"/>
-    <hyperlink r:id="rId30" ref="C85"/>
-    <hyperlink r:id="rId30" ref="C86"/>
-    <hyperlink r:id="rId34" ref="C87"/>
-    <hyperlink r:id="rId18" ref="C88"/>
-    <hyperlink r:id="rId20" ref="C89"/>
-    <hyperlink r:id="rId35" ref="C90"/>
-    <hyperlink r:id="rId7" ref="C91"/>
-    <hyperlink r:id="rId36" ref="C92"/>
-    <hyperlink r:id="rId37" ref="C93"/>
-    <hyperlink r:id="rId38" ref="C95"/>
-    <hyperlink r:id="rId7" ref="C96"/>
-    <hyperlink r:id="rId8" ref="C97"/>
-    <hyperlink r:id="rId39" ref="C99"/>
-    <hyperlink r:id="rId24" ref="C101"/>
-    <hyperlink r:id="rId32" ref="C102"/>
-    <hyperlink r:id="rId24" ref="C103"/>
-    <hyperlink r:id="rId40" ref="C104"/>
-    <hyperlink r:id="rId41" ref="C105"/>
-    <hyperlink r:id="rId42" ref="C106"/>
+    <hyperlink ref="C3" r:id="rId1"/>
+    <hyperlink ref="C4" r:id="rId2"/>
+    <hyperlink ref="C5" r:id="rId3"/>
+    <hyperlink ref="C6" r:id="rId4"/>
+    <hyperlink ref="C7" r:id="rId5"/>
+    <hyperlink ref="C8" r:id="rId6"/>
+    <hyperlink ref="C9" r:id="rId7"/>
+    <hyperlink ref="C10" r:id="rId8"/>
+    <hyperlink ref="C11" r:id="rId9"/>
+    <hyperlink ref="C12" r:id="rId10"/>
+    <hyperlink ref="C13" r:id="rId11"/>
+    <hyperlink ref="C14" r:id="rId12"/>
+    <hyperlink ref="C15" r:id="rId13"/>
+    <hyperlink ref="C16" r:id="rId14"/>
+    <hyperlink ref="C17" r:id="rId15"/>
+    <hyperlink ref="C18" r:id="rId16"/>
+    <hyperlink ref="C19" r:id="rId17"/>
+    <hyperlink ref="C20" r:id="rId18"/>
+    <hyperlink ref="C21" r:id="rId19"/>
+    <hyperlink ref="C22" r:id="rId20"/>
+    <hyperlink ref="C23" r:id="rId21"/>
+    <hyperlink ref="C24" r:id="rId22"/>
+    <hyperlink ref="C25" r:id="rId23"/>
+    <hyperlink ref="C26" r:id="rId24"/>
+    <hyperlink ref="C27" r:id="rId25"/>
+    <hyperlink ref="C28" r:id="rId26"/>
+    <hyperlink ref="C29" r:id="rId27"/>
+    <hyperlink ref="C30" r:id="rId28"/>
+    <hyperlink ref="C31" r:id="rId29"/>
+    <hyperlink ref="C32" r:id="rId30"/>
+    <hyperlink ref="C33" r:id="rId31"/>
+    <hyperlink ref="C34" r:id="rId32"/>
+    <hyperlink ref="C35" r:id="rId33"/>
+    <hyperlink ref="C36" r:id="rId34"/>
+    <hyperlink ref="C37" r:id="rId35"/>
+    <hyperlink ref="C38" r:id="rId36"/>
+    <hyperlink ref="C39" r:id="rId37"/>
+    <hyperlink ref="C40" r:id="rId38"/>
+    <hyperlink ref="C41" r:id="rId39"/>
+    <hyperlink ref="C42" r:id="rId40"/>
+    <hyperlink ref="C43" r:id="rId41"/>
+    <hyperlink ref="C44" r:id="rId42"/>
+    <hyperlink ref="C45" r:id="rId43"/>
+    <hyperlink ref="C46" r:id="rId44"/>
+    <hyperlink ref="C47" r:id="rId45"/>
+    <hyperlink ref="C48" r:id="rId46"/>
+    <hyperlink ref="C49" r:id="rId47"/>
+    <hyperlink ref="C50" r:id="rId48"/>
+    <hyperlink ref="C51" r:id="rId49"/>
+    <hyperlink ref="C52" r:id="rId50"/>
+    <hyperlink ref="C53" r:id="rId51"/>
+    <hyperlink ref="C54" r:id="rId52"/>
+    <hyperlink ref="C55" r:id="rId53"/>
+    <hyperlink ref="C56" r:id="rId54"/>
+    <hyperlink ref="C57" r:id="rId55"/>
+    <hyperlink ref="C58" r:id="rId56"/>
+    <hyperlink ref="C59" r:id="rId57"/>
+    <hyperlink ref="C60" r:id="rId58"/>
+    <hyperlink ref="C62" r:id="rId59"/>
+    <hyperlink ref="C63" r:id="rId60"/>
+    <hyperlink ref="C64" r:id="rId61"/>
+    <hyperlink ref="C65" r:id="rId62"/>
+    <hyperlink ref="C66" r:id="rId63"/>
+    <hyperlink ref="C67" r:id="rId64"/>
+    <hyperlink ref="C68" r:id="rId65"/>
+    <hyperlink ref="C69" r:id="rId66"/>
+    <hyperlink ref="C70" r:id="rId67"/>
+    <hyperlink ref="C71" r:id="rId68"/>
+    <hyperlink ref="C72" r:id="rId69"/>
+    <hyperlink ref="C73" r:id="rId70"/>
+    <hyperlink ref="C74" r:id="rId71"/>
+    <hyperlink ref="C75" r:id="rId72"/>
+    <hyperlink ref="C76" r:id="rId73"/>
+    <hyperlink ref="C77" r:id="rId74"/>
+    <hyperlink ref="C78" r:id="rId75"/>
+    <hyperlink ref="C79" r:id="rId76"/>
+    <hyperlink ref="C80" r:id="rId77"/>
+    <hyperlink ref="C81" r:id="rId78"/>
+    <hyperlink ref="C82" r:id="rId79"/>
+    <hyperlink ref="C83" r:id="rId80"/>
+    <hyperlink ref="C84" r:id="rId81"/>
+    <hyperlink ref="C85" r:id="rId82"/>
+    <hyperlink ref="C86" r:id="rId83"/>
+    <hyperlink ref="C87" r:id="rId84"/>
+    <hyperlink ref="C88" r:id="rId85"/>
+    <hyperlink ref="C89" r:id="rId86"/>
+    <hyperlink ref="C90" r:id="rId87"/>
+    <hyperlink ref="C91" r:id="rId88"/>
+    <hyperlink ref="C92" r:id="rId89"/>
+    <hyperlink ref="C93" r:id="rId90"/>
+    <hyperlink ref="C95" r:id="rId91"/>
+    <hyperlink ref="C96" r:id="rId92"/>
+    <hyperlink ref="C97" r:id="rId93"/>
+    <hyperlink ref="C99" r:id="rId94"/>
+    <hyperlink ref="C101" r:id="rId95"/>
+    <hyperlink ref="C102" r:id="rId96"/>
+    <hyperlink ref="C103" r:id="rId97"/>
+    <hyperlink ref="C104" r:id="rId98"/>
+    <hyperlink ref="C105" r:id="rId99"/>
+    <hyperlink ref="C106" r:id="rId100"/>
   </hyperlinks>
-  <printOptions headings="0" gridLines="0" horizontalCentered="0" verticalCentered="0"/>
-  <pageMargins left="0.78750000000000009" right="0.78750000000000009" top="1.05277777777778" bottom="1.05277777777778" header="0.78750000000000009" footer="0.78750000000000009"/>
-  <pageSetup paperSize="1" scale="100" firstPageNumber="1" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="1" errors="displayed" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageMargins left="0.7875000000000001" right="0.7875000000000001" top="1.05277777777778" bottom="1.05277777777778" header="0.7875000000000001" footer="0.7875000000000001"/>
+  <pageSetup paperSize="1" orientation="portrait" horizontalDpi="300" verticalDpi="300" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" usePrinterDefaults="1" copies="1"/>
   <headerFooter>
     <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;A</oddHeader>
     <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12Page &amp;P</oddFooter>

</xml_diff>